<commit_message>
📊 BIST Screener | 06.05.2026 16:30 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-06.xlsx
+++ b/data/bist_screener_2026-05-06.xlsx
@@ -6055,44 +6055,38 @@
     <row r="129">
       <c r="A129" s="6" t="inlineStr">
         <is>
-          <t>KCHOL</t>
+          <t>SASA</t>
         </is>
       </c>
       <c r="B129" s="7" t="n">
-        <v>210.5</v>
+        <v>3.08</v>
       </c>
       <c r="C129" s="8" t="n">
-        <v>0.0426</v>
+        <v>0.0301</v>
       </c>
       <c r="D129" s="9" t="n">
-        <v>18460000</v>
+        <v>5190000000</v>
       </c>
       <c r="E129" s="8" t="n">
-        <v>0.3672</v>
+        <v>0.3118</v>
       </c>
       <c r="F129" s="7" t="n">
-        <v>60.11</v>
-      </c>
-      <c r="G129" s="7" t="n">
-        <v>24.69</v>
-      </c>
+        <v>59.05</v>
+      </c>
+      <c r="G129" s="6" t="inlineStr"/>
       <c r="H129" s="7" t="n">
         <v>0.79</v>
       </c>
-      <c r="I129" s="8" t="n">
-        <v>0.0358</v>
-      </c>
-      <c r="J129" s="8" t="n">
-        <v>-0.0001</v>
-      </c>
+      <c r="I129" s="6" t="inlineStr"/>
+      <c r="J129" s="6" t="inlineStr"/>
       <c r="K129" s="6" t="inlineStr">
         <is>
-          <t>Enerji mineralleri</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L129" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HOLDING VE YATIRIM, BIST 50, BIST MALİ, BIST İSTANBUL, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST BANKA DISI LIKIT 10, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500, STOXX Eastern Europe 50</t>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST 50, BIST KİMYA PETROL PLASTİK, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST BANKA DISI LIKIT 10, BIST SÜRDÜRÜLEBİLİRLİK, ADANA, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M129" s="6" t="inlineStr"/>
@@ -6100,44 +6094,44 @@
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>PGSUS</t>
+          <t>KCHOL</t>
         </is>
       </c>
       <c r="B130" s="3" t="n">
-        <v>184.3</v>
+        <v>210.5</v>
       </c>
       <c r="C130" s="4" t="n">
-        <v>0.0313</v>
+        <v>0.0426</v>
       </c>
       <c r="D130" s="5" t="n">
-        <v>12270000</v>
+        <v>18460000</v>
       </c>
       <c r="E130" s="4" t="n">
-        <v>0.4568</v>
+        <v>0.3672</v>
       </c>
       <c r="F130" s="3" t="n">
-        <v>50.21</v>
+        <v>60.11</v>
       </c>
       <c r="G130" s="3" t="n">
-        <v>6.7</v>
+        <v>24.69</v>
       </c>
       <c r="H130" s="3" t="n">
         <v>0.79</v>
       </c>
       <c r="I130" s="4" t="n">
-        <v>0.1434</v>
+        <v>0.0358</v>
       </c>
       <c r="J130" s="4" t="n">
-        <v>-0.9609000000000001</v>
+        <v>-0.0001</v>
       </c>
       <c r="K130" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
+          <t>Enerji mineralleri</t>
         </is>
       </c>
       <c r="L130" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST ULASTIRMA, BIST TÜM, BIST 50, BIST HİZMETLER, BIST İSTANBUL, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST BANKA DISI LIKIT 10, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HOLDING VE YATIRIM, BIST 50, BIST MALİ, BIST İSTANBUL, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST BANKA DISI LIKIT 10, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500, STOXX Eastern Europe 50</t>
         </is>
       </c>
       <c r="M130" s="2" t="inlineStr"/>
@@ -6145,44 +6139,44 @@
     <row r="131">
       <c r="A131" s="6" t="inlineStr">
         <is>
-          <t>GOKNR</t>
+          <t>PGSUS</t>
         </is>
       </c>
       <c r="B131" s="7" t="n">
-        <v>21.94</v>
+        <v>184.3</v>
       </c>
       <c r="C131" s="8" t="n">
-        <v>0.0262</v>
+        <v>0.0313</v>
       </c>
       <c r="D131" s="9" t="n">
-        <v>4990000</v>
+        <v>12270000</v>
       </c>
       <c r="E131" s="8" t="n">
-        <v>0.2656</v>
+        <v>0.4568</v>
       </c>
       <c r="F131" s="7" t="n">
-        <v>49.87</v>
+        <v>50.21</v>
       </c>
       <c r="G131" s="7" t="n">
-        <v>18.58</v>
+        <v>6.7</v>
       </c>
       <c r="H131" s="7" t="n">
         <v>0.79</v>
       </c>
       <c r="I131" s="8" t="n">
-        <v>0.0488</v>
+        <v>0.1434</v>
       </c>
       <c r="J131" s="8" t="n">
-        <v>-3.3307</v>
+        <v>-0.9609000000000001</v>
       </c>
       <c r="K131" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Taşımacılık</t>
         </is>
       </c>
       <c r="L131" s="6" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST ULASTIRMA, BIST TÜM, BIST 50, BIST HİZMETLER, BIST İSTANBUL, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST BANKA DISI LIKIT 10, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M131" s="6" t="inlineStr"/>
@@ -6190,42 +6184,44 @@
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>ATAGY</t>
+          <t>GOKNR</t>
         </is>
       </c>
       <c r="B132" s="3" t="n">
-        <v>13.18</v>
+        <v>21.94</v>
       </c>
       <c r="C132" s="4" t="n">
-        <v>0.0023</v>
+        <v>0.0262</v>
       </c>
       <c r="D132" s="5" t="n">
-        <v>249260</v>
+        <v>4990000</v>
       </c>
       <c r="E132" s="4" t="n">
-        <v>0.6889</v>
+        <v>0.2656</v>
       </c>
       <c r="F132" s="3" t="n">
-        <v>56.05</v>
-      </c>
-      <c r="G132" s="2" t="inlineStr"/>
+        <v>49.87</v>
+      </c>
+      <c r="G132" s="3" t="n">
+        <v>18.58</v>
+      </c>
       <c r="H132" s="3" t="n">
         <v>0.79</v>
       </c>
       <c r="I132" s="4" t="n">
-        <v>-0.0266</v>
+        <v>0.0488</v>
       </c>
       <c r="J132" s="4" t="n">
-        <v>-0.5014999999999999</v>
+        <v>-3.3307</v>
       </c>
       <c r="K132" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L132" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M132" s="2" t="inlineStr"/>
@@ -6233,42 +6229,42 @@
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
         <is>
-          <t>BLCYT</t>
+          <t>ATAGY</t>
         </is>
       </c>
       <c r="B133" s="7" t="n">
-        <v>33.62</v>
+        <v>13.18</v>
       </c>
       <c r="C133" s="8" t="n">
-        <v>0.0313</v>
+        <v>0.0023</v>
       </c>
       <c r="D133" s="9" t="n">
-        <v>3360000</v>
+        <v>249260</v>
       </c>
       <c r="E133" s="8" t="n">
-        <v>0.3318</v>
+        <v>0.6889</v>
       </c>
       <c r="F133" s="7" t="n">
-        <v>39.94</v>
-      </c>
-      <c r="G133" s="7" t="n">
-        <v>88.92</v>
-      </c>
+        <v>56.05</v>
+      </c>
+      <c r="G133" s="6" t="inlineStr"/>
       <c r="H133" s="7" t="n">
         <v>0.79</v>
       </c>
       <c r="I133" s="8" t="n">
-        <v>0.0159</v>
-      </c>
-      <c r="J133" s="6" t="inlineStr"/>
+        <v>-0.0266</v>
+      </c>
+      <c r="J133" s="8" t="n">
+        <v>-0.5014999999999999</v>
+      </c>
       <c r="K133" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L133" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST ANA, ADANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ</t>
         </is>
       </c>
       <c r="M133" s="6" t="inlineStr"/>
@@ -6276,44 +6272,42 @@
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>PRDGS</t>
+          <t>BLCYT</t>
         </is>
       </c>
       <c r="B134" s="3" t="n">
-        <v>9.300000000000001</v>
+        <v>33.62</v>
       </c>
       <c r="C134" s="4" t="n">
-        <v>0.0941</v>
+        <v>0.0313</v>
       </c>
       <c r="D134" s="5" t="n">
-        <v>16710000</v>
+        <v>3360000</v>
       </c>
       <c r="E134" s="4" t="n">
-        <v>0.5656</v>
+        <v>0.3318</v>
       </c>
       <c r="F134" s="3" t="n">
-        <v>69.31999999999999</v>
+        <v>39.94</v>
       </c>
       <c r="G134" s="3" t="n">
-        <v>38.72</v>
+        <v>88.92</v>
       </c>
       <c r="H134" s="3" t="n">
-        <v>0.8</v>
+        <v>0.79</v>
       </c>
       <c r="I134" s="4" t="n">
-        <v>0.0237</v>
-      </c>
-      <c r="J134" s="4" t="n">
-        <v>2.8244</v>
-      </c>
+        <v>0.0159</v>
+      </c>
+      <c r="J134" s="2" t="inlineStr"/>
       <c r="K134" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L134" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST ANA, ADANA</t>
         </is>
       </c>
       <c r="M134" s="2" t="inlineStr"/>
@@ -6321,42 +6315,44 @@
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
         <is>
-          <t>SKTAS</t>
+          <t>PRDGS</t>
         </is>
       </c>
       <c r="B135" s="7" t="n">
-        <v>3.62</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="C135" s="8" t="n">
-        <v>0.0372</v>
-      </c>
-      <c r="D135" s="7" t="n">
-        <v>16620000</v>
+        <v>0.0941</v>
+      </c>
+      <c r="D135" s="9" t="n">
+        <v>16710000</v>
       </c>
       <c r="E135" s="8" t="n">
-        <v>0.5995</v>
+        <v>0.5656</v>
       </c>
       <c r="F135" s="7" t="n">
-        <v>64.58</v>
-      </c>
-      <c r="G135" s="6" t="inlineStr"/>
+        <v>69.31999999999999</v>
+      </c>
+      <c r="G135" s="7" t="n">
+        <v>38.72</v>
+      </c>
       <c r="H135" s="7" t="n">
         <v>0.8</v>
       </c>
       <c r="I135" s="8" t="n">
-        <v>-0.1172</v>
+        <v>0.0237</v>
       </c>
       <c r="J135" s="8" t="n">
-        <v>-4.7257</v>
+        <v>2.8244</v>
       </c>
       <c r="K135" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L135" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST ANA, BIST AYDIN</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M135" s="6" t="inlineStr"/>
@@ -6364,44 +6360,42 @@
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>TMSN</t>
+          <t>SKTAS</t>
         </is>
       </c>
       <c r="B136" s="3" t="n">
-        <v>104</v>
+        <v>3.62</v>
       </c>
       <c r="C136" s="4" t="n">
-        <v>-0.0029</v>
-      </c>
-      <c r="D136" s="5" t="n">
-        <v>873530</v>
+        <v>0.0372</v>
+      </c>
+      <c r="D136" s="3" t="n">
+        <v>16620000</v>
       </c>
       <c r="E136" s="4" t="n">
-        <v>0.287</v>
+        <v>0.5995</v>
       </c>
       <c r="F136" s="3" t="n">
-        <v>50.91</v>
-      </c>
-      <c r="G136" s="3" t="n">
-        <v>3.89</v>
-      </c>
+        <v>64.58</v>
+      </c>
+      <c r="G136" s="2" t="inlineStr"/>
       <c r="H136" s="3" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="I136" s="4" t="n">
-        <v>0.2876</v>
+        <v>-0.1172</v>
       </c>
       <c r="J136" s="4" t="n">
-        <v>-8.504899999999999</v>
+        <v>-4.7257</v>
       </c>
       <c r="K136" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L136" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST YILDIZ, BIST KONYA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TEKSTİL DERİ, BIST ANA, BIST AYDIN</t>
         </is>
       </c>
       <c r="M136" s="2" t="inlineStr"/>
@@ -6409,44 +6403,44 @@
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
         <is>
-          <t>PAGYO</t>
+          <t>TMSN</t>
         </is>
       </c>
       <c r="B137" s="7" t="n">
-        <v>141.2</v>
+        <v>104</v>
       </c>
       <c r="C137" s="8" t="n">
-        <v>0.09970000000000001</v>
+        <v>-0.0029</v>
       </c>
       <c r="D137" s="9" t="n">
-        <v>252810</v>
+        <v>873530</v>
       </c>
       <c r="E137" s="8" t="n">
-        <v>0.6475</v>
+        <v>0.287</v>
       </c>
       <c r="F137" s="7" t="n">
-        <v>66.42</v>
+        <v>50.91</v>
       </c>
       <c r="G137" s="7" t="n">
-        <v>7.96</v>
+        <v>3.89</v>
       </c>
       <c r="H137" s="7" t="n">
         <v>0.8100000000000001</v>
       </c>
       <c r="I137" s="8" t="n">
-        <v>0.1188</v>
+        <v>0.2876</v>
       </c>
       <c r="J137" s="8" t="n">
-        <v>5.5933</v>
+        <v>-8.504899999999999</v>
       </c>
       <c r="K137" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L137" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ESYA MAKİNA, BIST YILDIZ, BIST KONYA</t>
         </is>
       </c>
       <c r="M137" s="6" t="inlineStr"/>
@@ -6454,42 +6448,44 @@
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>CEMTS</t>
+          <t>PAGYO</t>
         </is>
       </c>
       <c r="B138" s="3" t="n">
-        <v>10.87</v>
+        <v>141.2</v>
       </c>
       <c r="C138" s="4" t="n">
-        <v>0.0178</v>
+        <v>0.09970000000000001</v>
       </c>
       <c r="D138" s="5" t="n">
-        <v>3400000</v>
+        <v>252810</v>
       </c>
       <c r="E138" s="4" t="n">
-        <v>0.3352000000000001</v>
+        <v>0.6475</v>
       </c>
       <c r="F138" s="3" t="n">
-        <v>48.71</v>
-      </c>
-      <c r="G138" s="2" t="inlineStr"/>
+        <v>66.42</v>
+      </c>
+      <c r="G138" s="3" t="n">
+        <v>7.96</v>
+      </c>
       <c r="H138" s="3" t="n">
-        <v>0.83</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="I138" s="4" t="n">
-        <v>-0.0184</v>
+        <v>0.1188</v>
       </c>
       <c r="J138" s="4" t="n">
-        <v>-18.3247</v>
+        <v>5.5933</v>
       </c>
       <c r="K138" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L138" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST BURSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M138" s="2" t="inlineStr"/>
@@ -6497,44 +6493,42 @@
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
         <is>
-          <t>A1CAP</t>
+          <t>CEMTS</t>
         </is>
       </c>
       <c r="B139" s="7" t="n">
-        <v>11.5</v>
+        <v>10.87</v>
       </c>
       <c r="C139" s="8" t="n">
-        <v>0.0026</v>
+        <v>0.0178</v>
       </c>
       <c r="D139" s="9" t="n">
-        <v>18950000</v>
+        <v>3400000</v>
       </c>
       <c r="E139" s="8" t="n">
-        <v>0.7115</v>
+        <v>0.3352000000000001</v>
       </c>
       <c r="F139" s="7" t="n">
-        <v>27.28</v>
-      </c>
-      <c r="G139" s="7" t="n">
-        <v>2.08</v>
-      </c>
+        <v>48.71</v>
+      </c>
+      <c r="G139" s="6" t="inlineStr"/>
       <c r="H139" s="7" t="n">
-        <v>0.85</v>
+        <v>0.83</v>
       </c>
       <c r="I139" s="8" t="n">
-        <v>0.5625</v>
+        <v>-0.0184</v>
       </c>
       <c r="J139" s="8" t="n">
-        <v>4.1559</v>
+        <v>-18.3247</v>
       </c>
       <c r="K139" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L139" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ARACI KURUMLAR, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST BURSA</t>
         </is>
       </c>
       <c r="M139" s="6" t="inlineStr"/>
@@ -6542,35 +6536,35 @@
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>ISCTR</t>
+          <t>A1CAP</t>
         </is>
       </c>
       <c r="B140" s="3" t="n">
-        <v>14.49</v>
+        <v>11.5</v>
       </c>
       <c r="C140" s="4" t="n">
-        <v>0.0343</v>
+        <v>0.0026</v>
       </c>
       <c r="D140" s="5" t="n">
-        <v>526220000</v>
+        <v>18950000</v>
       </c>
       <c r="E140" s="4" t="n">
-        <v>0.3325</v>
+        <v>0.7115</v>
       </c>
       <c r="F140" s="3" t="n">
-        <v>52.9</v>
+        <v>27.28</v>
       </c>
       <c r="G140" s="3" t="n">
-        <v>5.34</v>
+        <v>2.08</v>
       </c>
       <c r="H140" s="3" t="n">
         <v>0.85</v>
       </c>
       <c r="I140" s="4" t="n">
-        <v>0.1819</v>
+        <v>0.5625</v>
       </c>
       <c r="J140" s="4" t="n">
-        <v>0.6855</v>
+        <v>4.1559</v>
       </c>
       <c r="K140" s="2" t="inlineStr">
         <is>
@@ -6579,7 +6573,7 @@
       </c>
       <c r="L140" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST BANKA, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST 50, BIST LİKİT BANKA, BIST MALİ, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500, STOXX Eastern Europe 50</t>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ARACI KURUMLAR, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M140" s="2" t="inlineStr"/>
@@ -6587,44 +6581,44 @@
     <row r="141">
       <c r="A141" s="6" t="inlineStr">
         <is>
-          <t>YYLGD</t>
+          <t>ISCTR</t>
         </is>
       </c>
       <c r="B141" s="7" t="n">
-        <v>12.38</v>
+        <v>14.49</v>
       </c>
       <c r="C141" s="8" t="n">
-        <v>0.0231</v>
+        <v>0.0343</v>
       </c>
       <c r="D141" s="9" t="n">
-        <v>9560000</v>
+        <v>526220000</v>
       </c>
       <c r="E141" s="8" t="n">
-        <v>0.9348000000000001</v>
+        <v>0.3325</v>
       </c>
       <c r="F141" s="7" t="n">
-        <v>61.72</v>
+        <v>52.9</v>
       </c>
       <c r="G141" s="7" t="n">
-        <v>16.86</v>
+        <v>5.34</v>
       </c>
       <c r="H141" s="7" t="n">
         <v>0.85</v>
       </c>
       <c r="I141" s="8" t="n">
-        <v>0.0588</v>
+        <v>0.1819</v>
       </c>
       <c r="J141" s="8" t="n">
-        <v>11.314</v>
+        <v>0.6855</v>
       </c>
       <c r="K141" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L141" s="6" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST YILDIZ, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST 100, BIST 30, BIST BANKA, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST 50, BIST LİKİT BANKA, BIST MALİ, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500, STOXX Eastern Europe 50</t>
         </is>
       </c>
       <c r="M141" s="6" t="inlineStr"/>
@@ -6632,122 +6626,124 @@
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>BRKO</t>
+          <t>YYLGD</t>
         </is>
       </c>
       <c r="B142" s="3" t="n">
-        <v>13</v>
+        <v>12.38</v>
       </c>
       <c r="C142" s="4" t="n">
-        <v>-0.0262</v>
+        <v>0.0231</v>
       </c>
       <c r="D142" s="5" t="n">
-        <v>625790</v>
-      </c>
-      <c r="E142" s="2" t="inlineStr"/>
+        <v>9560000</v>
+      </c>
+      <c r="E142" s="4" t="n">
+        <v>0.9348000000000001</v>
+      </c>
       <c r="F142" s="3" t="n">
-        <v>43.3</v>
+        <v>61.72</v>
       </c>
       <c r="G142" s="3" t="n">
-        <v>13.02</v>
+        <v>16.86</v>
       </c>
       <c r="H142" s="3" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="I142" s="4" t="n">
-        <v>0.07679999999999999</v>
-      </c>
-      <c r="J142" s="2" t="inlineStr"/>
+        <v>0.0588</v>
+      </c>
+      <c r="J142" s="4" t="n">
+        <v>11.314</v>
+      </c>
       <c r="K142" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
-        </is>
-      </c>
-      <c r="L142" s="2" t="inlineStr"/>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST YILDIZ, BIST KURUMSAL YÖNETİM</t>
+        </is>
+      </c>
       <c r="M142" s="2" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="6" t="inlineStr">
         <is>
-          <t>EREGL</t>
+          <t>BRKO</t>
         </is>
       </c>
       <c r="B143" s="7" t="n">
-        <v>37.68</v>
+        <v>13</v>
       </c>
       <c r="C143" s="8" t="n">
-        <v>0.0124</v>
+        <v>-0.0262</v>
       </c>
       <c r="D143" s="9" t="n">
-        <v>195730000</v>
-      </c>
-      <c r="E143" s="8" t="n">
-        <v>0.4648</v>
-      </c>
+        <v>625790</v>
+      </c>
+      <c r="E143" s="6" t="inlineStr"/>
       <c r="F143" s="7" t="n">
-        <v>75.33</v>
+        <v>43.3</v>
       </c>
       <c r="G143" s="7" t="n">
-        <v>539.83</v>
+        <v>13.02</v>
       </c>
       <c r="H143" s="7" t="n">
         <v>0.86</v>
       </c>
       <c r="I143" s="8" t="n">
-        <v>0.0017</v>
+        <v>0.07679999999999999</v>
       </c>
       <c r="J143" s="6" t="inlineStr"/>
       <c r="K143" s="6" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
-        </is>
-      </c>
-      <c r="L143" s="6" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST 50, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST BANKA DISI LIKIT 10, BIST TEMETTU, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM 30, BIST KATILIM TEMETTU, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500, STOXX Eastern Europe 50</t>
-        </is>
-      </c>
+          <t>Dayanıklı tüketim malları</t>
+        </is>
+      </c>
+      <c r="L143" s="6" t="inlineStr"/>
       <c r="M143" s="6" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>UNLU</t>
+          <t>EREGL</t>
         </is>
       </c>
       <c r="B144" s="3" t="n">
-        <v>13.94</v>
+        <v>37.68</v>
       </c>
       <c r="C144" s="4" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="D144" s="3" t="n">
-        <v>2090000</v>
+        <v>0.0124</v>
+      </c>
+      <c r="D144" s="5" t="n">
+        <v>195730000</v>
       </c>
       <c r="E144" s="4" t="n">
-        <v>0.3557</v>
+        <v>0.4648</v>
       </c>
       <c r="F144" s="3" t="n">
-        <v>56.37</v>
-      </c>
-      <c r="G144" s="2" t="inlineStr"/>
+        <v>75.33</v>
+      </c>
+      <c r="G144" s="3" t="n">
+        <v>539.83</v>
+      </c>
       <c r="H144" s="3" t="n">
-        <v>0.87</v>
+        <v>0.86</v>
       </c>
       <c r="I144" s="4" t="n">
-        <v>-0.0721</v>
-      </c>
-      <c r="J144" s="4" t="n">
-        <v>0.7347</v>
-      </c>
+        <v>0.0017</v>
+      </c>
+      <c r="J144" s="2" t="inlineStr"/>
       <c r="K144" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L144" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST METAL ANA, BIST 50, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST BANKA DISI LIKIT 10, BIST TEMETTU, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KATILIM 30, BIST KATILIM TEMETTU, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500, STOXX Eastern Europe 50</t>
         </is>
       </c>
       <c r="M144" s="2" t="inlineStr"/>
@@ -6755,42 +6751,42 @@
     <row r="145">
       <c r="A145" s="6" t="inlineStr">
         <is>
-          <t>SASA</t>
+          <t>UNLU</t>
         </is>
       </c>
       <c r="B145" s="7" t="n">
-        <v>3.08</v>
+        <v>13.94</v>
       </c>
       <c r="C145" s="8" t="n">
-        <v>0.0301</v>
-      </c>
-      <c r="D145" s="9" t="n">
-        <v>5190000000</v>
+        <v>0.025</v>
+      </c>
+      <c r="D145" s="7" t="n">
+        <v>2090000</v>
       </c>
       <c r="E145" s="8" t="n">
-        <v>0.3118</v>
+        <v>0.3557</v>
       </c>
       <c r="F145" s="7" t="n">
-        <v>59.05</v>
+        <v>56.37</v>
       </c>
       <c r="G145" s="6" t="inlineStr"/>
       <c r="H145" s="7" t="n">
         <v>0.87</v>
       </c>
       <c r="I145" s="8" t="n">
-        <v>-0.1556</v>
+        <v>-0.0721</v>
       </c>
       <c r="J145" s="8" t="n">
-        <v>-18.749</v>
+        <v>0.7347</v>
       </c>
       <c r="K145" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L145" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST 50, BIST KİMYA PETROL PLASTİK, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST BANKA DISI LIKIT 10, BIST SÜRDÜRÜLEBİLİRLİK, ADANA, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M145" s="6" t="inlineStr"/>
@@ -10908,44 +10904,44 @@
     <row r="240">
       <c r="A240" s="2" t="inlineStr">
         <is>
-          <t>TAVHL</t>
+          <t>TUREX</t>
         </is>
       </c>
       <c r="B240" s="3" t="n">
-        <v>289.75</v>
+        <v>9.08</v>
       </c>
       <c r="C240" s="4" t="n">
-        <v>0.0498</v>
+        <v>-0.005500000000000001</v>
       </c>
       <c r="D240" s="5" t="n">
-        <v>3660000</v>
+        <v>42390000</v>
       </c>
       <c r="E240" s="4" t="n">
-        <v>0.4979</v>
+        <v>0.4</v>
       </c>
       <c r="F240" s="3" t="n">
-        <v>43.38</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G240" s="3" t="n">
-        <v>37.38</v>
+        <v>16.17</v>
       </c>
       <c r="H240" s="3" t="n">
-        <v>1.32</v>
+        <v>1.33</v>
       </c>
       <c r="I240" s="4" t="n">
-        <v>0.0408</v>
+        <v>0.09420000000000001</v>
       </c>
       <c r="J240" s="4" t="n">
-        <v>-1.203</v>
+        <v>-0.8061</v>
       </c>
       <c r="K240" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L240" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HOLDING VE YATIRIM, BIST 50, BIST MALİ, BIST İSTANBUL, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST ULASTIRMA, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M240" s="2" t="inlineStr"/>
@@ -10953,44 +10949,44 @@
     <row r="241">
       <c r="A241" s="6" t="inlineStr">
         <is>
-          <t>TUREX</t>
+          <t>MARBL</t>
         </is>
       </c>
       <c r="B241" s="7" t="n">
-        <v>9.08</v>
+        <v>14.02</v>
       </c>
       <c r="C241" s="8" t="n">
-        <v>-0.005500000000000001</v>
+        <v>0.0086</v>
       </c>
       <c r="D241" s="9" t="n">
-        <v>42390000</v>
+        <v>4560000</v>
       </c>
       <c r="E241" s="8" t="n">
-        <v>0.4</v>
+        <v>0.2623</v>
       </c>
       <c r="F241" s="7" t="n">
-        <v>64.09999999999999</v>
+        <v>59.73</v>
       </c>
       <c r="G241" s="7" t="n">
-        <v>16.17</v>
+        <v>2696.15</v>
       </c>
       <c r="H241" s="7" t="n">
-        <v>1.33</v>
+        <v>1.35</v>
       </c>
       <c r="I241" s="8" t="n">
-        <v>0.09420000000000001</v>
+        <v>0.0005</v>
       </c>
       <c r="J241" s="8" t="n">
-        <v>-0.8061</v>
+        <v>-5.5053</v>
       </c>
       <c r="K241" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L241" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST ULASTIRMA, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M241" s="6" t="inlineStr"/>
@@ -10998,44 +10994,44 @@
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
         <is>
-          <t>MARBL</t>
+          <t>SURGY</t>
         </is>
       </c>
       <c r="B242" s="3" t="n">
-        <v>14.02</v>
+        <v>73</v>
       </c>
       <c r="C242" s="4" t="n">
-        <v>0.0086</v>
+        <v>-0.0234</v>
       </c>
       <c r="D242" s="5" t="n">
-        <v>4560000</v>
+        <v>9590000</v>
       </c>
       <c r="E242" s="4" t="n">
-        <v>0.2623</v>
+        <v>0.2449</v>
       </c>
       <c r="F242" s="3" t="n">
-        <v>59.73</v>
+        <v>64.39</v>
       </c>
       <c r="G242" s="3" t="n">
-        <v>2696.15</v>
+        <v>21.78</v>
       </c>
       <c r="H242" s="3" t="n">
         <v>1.35</v>
       </c>
       <c r="I242" s="4" t="n">
-        <v>0.0005</v>
+        <v>0.0737</v>
       </c>
       <c r="J242" s="4" t="n">
-        <v>-5.5053</v>
+        <v>-1.8749</v>
       </c>
       <c r="K242" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L242" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M242" s="2" t="inlineStr"/>
@@ -11043,36 +11039,34 @@
     <row r="243">
       <c r="A243" s="6" t="inlineStr">
         <is>
-          <t>SURGY</t>
+          <t>IHLGM</t>
         </is>
       </c>
       <c r="B243" s="7" t="n">
-        <v>73</v>
+        <v>2.35</v>
       </c>
       <c r="C243" s="8" t="n">
-        <v>-0.0234</v>
+        <v>0.0262</v>
       </c>
       <c r="D243" s="9" t="n">
-        <v>9590000</v>
+        <v>76960000</v>
       </c>
       <c r="E243" s="8" t="n">
-        <v>0.2449</v>
+        <v>0.7498999999999999</v>
       </c>
       <c r="F243" s="7" t="n">
-        <v>64.39</v>
+        <v>64.48</v>
       </c>
       <c r="G243" s="7" t="n">
-        <v>21.78</v>
+        <v>3.78</v>
       </c>
       <c r="H243" s="7" t="n">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="I243" s="8" t="n">
-        <v>0.0737</v>
-      </c>
-      <c r="J243" s="8" t="n">
-        <v>-1.8749</v>
-      </c>
+        <v>0.4857</v>
+      </c>
+      <c r="J243" s="6" t="inlineStr"/>
       <c r="K243" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -11080,7 +11074,7 @@
       </c>
       <c r="L243" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M243" s="6" t="inlineStr"/>
@@ -11088,42 +11082,44 @@
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
         <is>
-          <t>IHLGM</t>
+          <t>PINSU</t>
         </is>
       </c>
       <c r="B244" s="3" t="n">
-        <v>2.35</v>
+        <v>11.7</v>
       </c>
       <c r="C244" s="4" t="n">
-        <v>0.0262</v>
+        <v>0.0112</v>
       </c>
       <c r="D244" s="5" t="n">
-        <v>76960000</v>
+        <v>3180000</v>
       </c>
       <c r="E244" s="4" t="n">
-        <v>0.7498999999999999</v>
+        <v>0.3326</v>
       </c>
       <c r="F244" s="3" t="n">
-        <v>64.48</v>
+        <v>46.98</v>
       </c>
       <c r="G244" s="3" t="n">
-        <v>3.78</v>
+        <v>345.13</v>
       </c>
       <c r="H244" s="3" t="n">
         <v>1.36</v>
       </c>
       <c r="I244" s="4" t="n">
-        <v>0.4857</v>
-      </c>
-      <c r="J244" s="2" t="inlineStr"/>
+        <v>0.0044</v>
+      </c>
+      <c r="J244" s="4" t="n">
+        <v>-1.293</v>
+      </c>
       <c r="K244" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L244" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST KURUMSAL YÖNETİM, BIST İZMİR</t>
         </is>
       </c>
       <c r="M244" s="2" t="inlineStr"/>
@@ -11131,44 +11127,44 @@
     <row r="245">
       <c r="A245" s="6" t="inlineStr">
         <is>
-          <t>PINSU</t>
+          <t>OYYAT</t>
         </is>
       </c>
       <c r="B245" s="7" t="n">
-        <v>11.7</v>
+        <v>55.05</v>
       </c>
       <c r="C245" s="8" t="n">
-        <v>0.0112</v>
+        <v>-0.08019999999999999</v>
       </c>
       <c r="D245" s="9" t="n">
-        <v>3180000</v>
+        <v>606020</v>
       </c>
       <c r="E245" s="8" t="n">
-        <v>0.3326</v>
+        <v>0.3035</v>
       </c>
       <c r="F245" s="7" t="n">
-        <v>46.98</v>
+        <v>45.72</v>
       </c>
       <c r="G245" s="7" t="n">
-        <v>345.13</v>
+        <v>7.26</v>
       </c>
       <c r="H245" s="7" t="n">
         <v>1.36</v>
       </c>
       <c r="I245" s="8" t="n">
-        <v>0.0044</v>
+        <v>0.231</v>
       </c>
       <c r="J245" s="8" t="n">
-        <v>-1.293</v>
+        <v>13.7151</v>
       </c>
       <c r="K245" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L245" s="6" t="inlineStr">
         <is>
-          <t>BIST GIDA ICECEK, BIST TUM-100, BIST SINAI, BIST TÜM, BIST ANA, BIST KURUMSAL YÖNETİM, BIST İZMİR</t>
+          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ARACI KURUMLAR, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M245" s="6" t="inlineStr"/>
@@ -11176,44 +11172,40 @@
     <row r="246">
       <c r="A246" s="2" t="inlineStr">
         <is>
-          <t>OYYAT</t>
+          <t>TAVHL</t>
         </is>
       </c>
       <c r="B246" s="3" t="n">
-        <v>55.05</v>
+        <v>289.75</v>
       </c>
       <c r="C246" s="4" t="n">
-        <v>-0.08019999999999999</v>
+        <v>0.0498</v>
       </c>
       <c r="D246" s="5" t="n">
-        <v>606020</v>
+        <v>3660000</v>
       </c>
       <c r="E246" s="4" t="n">
-        <v>0.3035</v>
+        <v>0.4979</v>
       </c>
       <c r="F246" s="3" t="n">
-        <v>45.72</v>
-      </c>
-      <c r="G246" s="3" t="n">
-        <v>7.26</v>
-      </c>
+        <v>43.38</v>
+      </c>
+      <c r="G246" s="2" t="inlineStr"/>
       <c r="H246" s="3" t="n">
         <v>1.36</v>
       </c>
-      <c r="I246" s="4" t="n">
-        <v>0.231</v>
-      </c>
+      <c r="I246" s="2" t="inlineStr"/>
       <c r="J246" s="4" t="n">
-        <v>13.7151</v>
+        <v>-1.474</v>
       </c>
       <c r="K246" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Taşımacılık</t>
         </is>
       </c>
       <c r="L246" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST MALİ, BIST ARACI KURUMLAR, BIST YILDIZ</t>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST HOLDING VE YATIRIM, BIST 50, BIST MALİ, BIST İSTANBUL, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST SÜRDÜRÜLEBİLİRLİK 25, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M246" s="2" t="inlineStr"/>
@@ -18267,40 +18259,40 @@
     <row r="409">
       <c r="A409" s="6" t="inlineStr">
         <is>
-          <t>ARFYE</t>
+          <t>CCOLA</t>
         </is>
       </c>
       <c r="B409" s="7" t="n">
-        <v>32.34</v>
+        <v>84.84999999999999</v>
       </c>
       <c r="C409" s="8" t="n">
-        <v>-0.0212</v>
+        <v>0.0626</v>
       </c>
       <c r="D409" s="9" t="n">
-        <v>8850000</v>
+        <v>6130000</v>
       </c>
       <c r="E409" s="8" t="n">
-        <v>0.2571</v>
+        <v>0.2895</v>
       </c>
       <c r="F409" s="7" t="n">
-        <v>58.92</v>
+        <v>71.62</v>
       </c>
       <c r="G409" s="6" t="inlineStr"/>
       <c r="H409" s="7" t="n">
-        <v>2.87</v>
+        <v>2.85</v>
       </c>
       <c r="I409" s="6" t="inlineStr"/>
       <c r="J409" s="8" t="n">
-        <v>-0.3467</v>
+        <v>689.6664999999999</v>
       </c>
       <c r="K409" s="6" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L409" s="6" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST 50, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST 50-30, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M409" s="6" t="inlineStr"/>
@@ -18308,42 +18300,40 @@
     <row r="410">
       <c r="A410" s="2" t="inlineStr">
         <is>
-          <t>VBTYZ</t>
+          <t>ARFYE</t>
         </is>
       </c>
       <c r="B410" s="3" t="n">
-        <v>22.52</v>
+        <v>32.34</v>
       </c>
       <c r="C410" s="4" t="n">
-        <v>-0.0268</v>
+        <v>-0.0212</v>
       </c>
       <c r="D410" s="5" t="n">
-        <v>1910000</v>
+        <v>8850000</v>
       </c>
       <c r="E410" s="4" t="n">
-        <v>0.371</v>
+        <v>0.2571</v>
       </c>
       <c r="F410" s="3" t="n">
-        <v>57.84</v>
-      </c>
-      <c r="G410" s="3" t="n">
-        <v>15.63</v>
-      </c>
+        <v>58.92</v>
+      </c>
+      <c r="G410" s="2" t="inlineStr"/>
       <c r="H410" s="3" t="n">
-        <v>2.89</v>
-      </c>
-      <c r="I410" s="4" t="n">
-        <v>0.2008</v>
-      </c>
-      <c r="J410" s="2" t="inlineStr"/>
+        <v>2.87</v>
+      </c>
+      <c r="I410" s="2" t="inlineStr"/>
+      <c r="J410" s="4" t="n">
+        <v>-0.3467</v>
+      </c>
       <c r="K410" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L410" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST KATILIM TÜM, BIST ANA, BIST İZMİR</t>
         </is>
       </c>
       <c r="M410" s="2" t="inlineStr"/>
@@ -18351,44 +18341,42 @@
     <row r="411">
       <c r="A411" s="6" t="inlineStr">
         <is>
-          <t>BIGCH</t>
+          <t>VBTYZ</t>
         </is>
       </c>
       <c r="B411" s="7" t="n">
-        <v>7.46</v>
+        <v>22.52</v>
       </c>
       <c r="C411" s="8" t="n">
-        <v>0.0054</v>
+        <v>-0.0268</v>
       </c>
       <c r="D411" s="9" t="n">
-        <v>8170000</v>
+        <v>1910000</v>
       </c>
       <c r="E411" s="8" t="n">
-        <v>0.4243</v>
+        <v>0.371</v>
       </c>
       <c r="F411" s="7" t="n">
-        <v>50.25</v>
+        <v>57.84</v>
       </c>
       <c r="G411" s="7" t="n">
-        <v>606.5</v>
+        <v>15.63</v>
       </c>
       <c r="H411" s="7" t="n">
-        <v>2.94</v>
+        <v>2.89</v>
       </c>
       <c r="I411" s="8" t="n">
-        <v>0.005</v>
-      </c>
-      <c r="J411" s="8" t="n">
-        <v>-2.3252</v>
-      </c>
+        <v>0.2008</v>
+      </c>
+      <c r="J411" s="6" t="inlineStr"/>
       <c r="K411" s="6" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L411" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TURİZM, BIST HİZMETLER, BIST İSTANBUL, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI</t>
         </is>
       </c>
       <c r="M411" s="6" t="inlineStr"/>
@@ -18396,40 +18384,44 @@
     <row r="412">
       <c r="A412" s="2" t="inlineStr">
         <is>
-          <t>ALFAS</t>
+          <t>BIGCH</t>
         </is>
       </c>
       <c r="B412" s="3" t="n">
-        <v>42.9</v>
+        <v>7.46</v>
       </c>
       <c r="C412" s="4" t="n">
-        <v>0.0317</v>
+        <v>0.0054</v>
       </c>
       <c r="D412" s="5" t="n">
-        <v>2620000</v>
+        <v>8170000</v>
       </c>
       <c r="E412" s="4" t="n">
-        <v>0.23</v>
+        <v>0.4243</v>
       </c>
       <c r="F412" s="3" t="n">
-        <v>70.73</v>
-      </c>
-      <c r="G412" s="2" t="inlineStr"/>
+        <v>50.25</v>
+      </c>
+      <c r="G412" s="3" t="n">
+        <v>606.5</v>
+      </c>
       <c r="H412" s="3" t="n">
-        <v>2.99</v>
+        <v>2.94</v>
       </c>
       <c r="I412" s="4" t="n">
-        <v>-0.0027</v>
-      </c>
-      <c r="J412" s="2" t="inlineStr"/>
+        <v>0.005</v>
+      </c>
+      <c r="J412" s="4" t="n">
+        <v>-2.3252</v>
+      </c>
       <c r="K412" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L412" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TURİZM, BIST HİZMETLER, BIST İSTANBUL, BIST ANA</t>
         </is>
       </c>
       <c r="M412" s="2" t="inlineStr"/>
@@ -18437,44 +18429,40 @@
     <row r="413">
       <c r="A413" s="6" t="inlineStr">
         <is>
-          <t>FONET</t>
+          <t>ALFAS</t>
         </is>
       </c>
       <c r="B413" s="7" t="n">
-        <v>5.42</v>
+        <v>42.9</v>
       </c>
       <c r="C413" s="8" t="n">
-        <v>-0.0109</v>
+        <v>0.0317</v>
       </c>
       <c r="D413" s="9" t="n">
-        <v>68890000</v>
+        <v>2620000</v>
       </c>
       <c r="E413" s="8" t="n">
-        <v>0.6164999999999999</v>
+        <v>0.23</v>
       </c>
       <c r="F413" s="7" t="n">
-        <v>63.91</v>
-      </c>
-      <c r="G413" s="7" t="n">
-        <v>23.04</v>
-      </c>
+        <v>70.73</v>
+      </c>
+      <c r="G413" s="6" t="inlineStr"/>
       <c r="H413" s="7" t="n">
-        <v>3</v>
+        <v>2.99</v>
       </c>
       <c r="I413" s="8" t="n">
-        <v>0.1565</v>
-      </c>
-      <c r="J413" s="8" t="n">
-        <v>0.7060999999999999</v>
-      </c>
+        <v>-0.0027</v>
+      </c>
+      <c r="J413" s="6" t="inlineStr"/>
       <c r="K413" s="6" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L413" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST ANKARA</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M413" s="6" t="inlineStr"/>
@@ -18482,44 +18470,44 @@
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
         <is>
-          <t>SUWEN</t>
+          <t>FONET</t>
         </is>
       </c>
       <c r="B414" s="3" t="n">
-        <v>8.92</v>
+        <v>5.42</v>
       </c>
       <c r="C414" s="4" t="n">
-        <v>0.0265</v>
+        <v>-0.0109</v>
       </c>
       <c r="D414" s="5" t="n">
-        <v>3350000</v>
+        <v>68890000</v>
       </c>
       <c r="E414" s="4" t="n">
-        <v>0.6501</v>
+        <v>0.6164999999999999</v>
       </c>
       <c r="F414" s="3" t="n">
-        <v>47.75</v>
+        <v>63.91</v>
       </c>
       <c r="G414" s="3" t="n">
-        <v>33.11</v>
+        <v>23.04</v>
       </c>
       <c r="H414" s="3" t="n">
-        <v>3.03</v>
+        <v>3</v>
       </c>
       <c r="I414" s="4" t="n">
-        <v>0.078</v>
+        <v>0.1565</v>
       </c>
       <c r="J414" s="4" t="n">
-        <v>-0.9328</v>
+        <v>0.7060999999999999</v>
       </c>
       <c r="K414" s="2" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L414" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST KATILIM 100, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST ANKARA</t>
         </is>
       </c>
       <c r="M414" s="2" t="inlineStr"/>
@@ -18527,124 +18515,126 @@
     <row r="415">
       <c r="A415" s="6" t="inlineStr">
         <is>
-          <t>CASA</t>
+          <t>SUWEN</t>
         </is>
       </c>
       <c r="B415" s="7" t="n">
-        <v>100</v>
+        <v>8.92</v>
       </c>
       <c r="C415" s="8" t="n">
-        <v>0.0741</v>
+        <v>0.0265</v>
       </c>
       <c r="D415" s="9" t="n">
-        <v>21840</v>
-      </c>
-      <c r="E415" s="6" t="inlineStr"/>
+        <v>3350000</v>
+      </c>
+      <c r="E415" s="8" t="n">
+        <v>0.6501</v>
+      </c>
       <c r="F415" s="7" t="n">
-        <v>56.71</v>
-      </c>
-      <c r="G415" s="6" t="inlineStr"/>
+        <v>47.75</v>
+      </c>
+      <c r="G415" s="7" t="n">
+        <v>33.11</v>
+      </c>
       <c r="H415" s="7" t="n">
-        <v>3.07</v>
+        <v>3.03</v>
       </c>
       <c r="I415" s="8" t="n">
-        <v>-0.6842</v>
+        <v>0.078</v>
       </c>
       <c r="J415" s="8" t="n">
-        <v>-193.4008</v>
+        <v>-0.9328</v>
       </c>
       <c r="K415" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L415" s="6" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L415" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST KATILIM TÜM, BIST YILDIZ, BIST TEMETTU, BIST KATILIM TEMETTU</t>
+        </is>
+      </c>
       <c r="M415" s="6" t="inlineStr"/>
     </row>
     <row r="416">
       <c r="A416" s="2" t="inlineStr">
         <is>
-          <t>TRALT</t>
+          <t>CASA</t>
         </is>
       </c>
       <c r="B416" s="3" t="n">
-        <v>42.06</v>
+        <v>100</v>
       </c>
       <c r="C416" s="4" t="n">
-        <v>0.0344</v>
+        <v>0.0741</v>
       </c>
       <c r="D416" s="5" t="n">
-        <v>115540000</v>
-      </c>
-      <c r="E416" s="4" t="n">
-        <v>0.3</v>
-      </c>
+        <v>21840</v>
+      </c>
+      <c r="E416" s="2" t="inlineStr"/>
       <c r="F416" s="3" t="n">
-        <v>42.37</v>
-      </c>
-      <c r="G416" s="3" t="n">
-        <v>34.2</v>
-      </c>
+        <v>56.71</v>
+      </c>
+      <c r="G416" s="2" t="inlineStr"/>
       <c r="H416" s="3" t="n">
-        <v>3.08</v>
+        <v>3.07</v>
       </c>
       <c r="I416" s="4" t="n">
-        <v>0.1092</v>
+        <v>-0.6842</v>
       </c>
       <c r="J416" s="4" t="n">
-        <v>-1.1669</v>
+        <v>-193.4008</v>
       </c>
       <c r="K416" s="2" t="inlineStr">
         <is>
-          <t>Enerji-dışı mineraller</t>
-        </is>
-      </c>
-      <c r="L416" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST 50, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST BANKA DISI LIKIT 10, BIST İZMİR, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
-        </is>
-      </c>
+          <t>Dağıtım servisleri</t>
+        </is>
+      </c>
+      <c r="L416" s="2" t="inlineStr"/>
       <c r="M416" s="2" t="inlineStr"/>
     </row>
     <row r="417">
       <c r="A417" s="6" t="inlineStr">
         <is>
-          <t>KMPUR</t>
+          <t>TRALT</t>
         </is>
       </c>
       <c r="B417" s="7" t="n">
-        <v>21.92</v>
+        <v>42.06</v>
       </c>
       <c r="C417" s="8" t="n">
-        <v>0.0148</v>
+        <v>0.0344</v>
       </c>
       <c r="D417" s="9" t="n">
-        <v>6530000</v>
+        <v>115540000</v>
       </c>
       <c r="E417" s="8" t="n">
-        <v>0.1951</v>
+        <v>0.3</v>
       </c>
       <c r="F417" s="7" t="n">
-        <v>72.3</v>
-      </c>
-      <c r="G417" s="6" t="inlineStr"/>
+        <v>42.37</v>
+      </c>
+      <c r="G417" s="7" t="n">
+        <v>34.2</v>
+      </c>
       <c r="H417" s="7" t="n">
-        <v>3.1</v>
+        <v>3.08</v>
       </c>
       <c r="I417" s="8" t="n">
-        <v>-0.098</v>
+        <v>0.1092</v>
       </c>
       <c r="J417" s="8" t="n">
-        <v>2.4746</v>
+        <v>-1.1669</v>
       </c>
       <c r="K417" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Enerji-dışı mineraller</t>
         </is>
       </c>
       <c r="L417" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KOCAELI, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
+          <t>BIST 100, BIST 30, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST SINAI, BIST TÜM, BIST MADENCİLİK, BIST 50, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST BANKA DISI LIKIT 10, BIST İZMİR, BIST 30 AĞIRLIK SINIRLAMALI 10, BIST 30 EŞİT AĞIRLIKLI GETİRİ, BIST 30 AĞIRLIK SINIRLAMALI 25, STOXX Emerging Markets 1500</t>
         </is>
       </c>
       <c r="M417" s="6" t="inlineStr"/>
@@ -18652,44 +18642,42 @@
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
         <is>
-          <t>GRSEL</t>
+          <t>KMPUR</t>
         </is>
       </c>
       <c r="B418" s="3" t="n">
-        <v>321</v>
+        <v>21.92</v>
       </c>
       <c r="C418" s="4" t="n">
-        <v>0.0682</v>
+        <v>0.0148</v>
       </c>
       <c r="D418" s="5" t="n">
-        <v>663010</v>
+        <v>6530000</v>
       </c>
       <c r="E418" s="4" t="n">
-        <v>0.2907</v>
+        <v>0.1951</v>
       </c>
       <c r="F418" s="3" t="n">
-        <v>55.01</v>
-      </c>
-      <c r="G418" s="3" t="n">
-        <v>11.82</v>
-      </c>
+        <v>72.3</v>
+      </c>
+      <c r="G418" s="2" t="inlineStr"/>
       <c r="H418" s="3" t="n">
-        <v>3.12</v>
+        <v>3.1</v>
       </c>
       <c r="I418" s="4" t="n">
-        <v>0.3345</v>
+        <v>-0.098</v>
       </c>
       <c r="J418" s="4" t="n">
-        <v>0.6006</v>
+        <v>2.4746</v>
       </c>
       <c r="K418" s="2" t="inlineStr">
         <is>
-          <t>Tüketici hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L418" s="2" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST ULASTIRMA, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KATILIM TEMETTU, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST KATILIM TÜM, BIST YILDIZ, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST KOCAELI, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
         </is>
       </c>
       <c r="M418" s="2" t="inlineStr"/>
@@ -18697,44 +18685,44 @@
     <row r="419">
       <c r="A419" s="6" t="inlineStr">
         <is>
-          <t>CCOLA</t>
+          <t>GRSEL</t>
         </is>
       </c>
       <c r="B419" s="7" t="n">
-        <v>84.84999999999999</v>
+        <v>321</v>
       </c>
       <c r="C419" s="8" t="n">
-        <v>0.0626</v>
+        <v>0.0682</v>
       </c>
       <c r="D419" s="9" t="n">
-        <v>6130000</v>
+        <v>663010</v>
       </c>
       <c r="E419" s="8" t="n">
-        <v>0.2895</v>
+        <v>0.2907</v>
       </c>
       <c r="F419" s="7" t="n">
-        <v>71.62</v>
+        <v>55.01</v>
       </c>
       <c r="G419" s="7" t="n">
-        <v>17.57</v>
+        <v>11.82</v>
       </c>
       <c r="H419" s="7" t="n">
-        <v>3.13</v>
+        <v>3.12</v>
       </c>
       <c r="I419" s="8" t="n">
-        <v>0.2087</v>
+        <v>0.3345</v>
       </c>
       <c r="J419" s="8" t="n">
-        <v>-0.9989</v>
+        <v>0.6006</v>
       </c>
       <c r="K419" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Tüketici hizmetleri</t>
         </is>
       </c>
       <c r="L419" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST GIDA ICECEK, BIST SINAI, BIST TÜM, BIST 50, BIST İSTANBUL, BIST 100-30, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU 25, BIST TEMETTU, BIST SÜRDÜRÜLEBİLİRLİK, BIST KURUMSAL YÖNETİM, BIST 50-30, BIST 50-30 AGIRLIK SINIRLAMALI 25, BIST 50-30 AĞIRLIK SINIRLAMALI 10, STOXX Emerging Markets 1500</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST ULASTIRMA, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST TEMETTU, BIST KATILIM 50, BIST SÜRDÜRÜLEBİLİRLİK, BIST KATILIM TEMETTU, BIST KATILIM SÜRDÜRÜLEBİLİRLİİK</t>
         </is>
       </c>
       <c r="M419" s="6" t="inlineStr"/>
@@ -25910,34 +25898,38 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>17.49</v>
+        <v>35.22</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>-0.0224</v>
-      </c>
-      <c r="D586" s="3" t="n">
-        <v>66930000.00000001</v>
-      </c>
-      <c r="E586" s="2" t="inlineStr"/>
+        <v>0.015</v>
+      </c>
+      <c r="D586" s="5" t="n">
+        <v>6830000</v>
+      </c>
+      <c r="E586" s="4" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F586" s="3" t="n">
-        <v>54.24</v>
+        <v>42.78</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
       <c r="I586" s="2" t="inlineStr"/>
-      <c r="J586" s="2" t="inlineStr"/>
+      <c r="J586" s="4" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25945,23 +25937,21 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>6.3</v>
+        <v>44</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0237</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>51450000</v>
-      </c>
-      <c r="E587" s="8" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>13410000</v>
+      </c>
+      <c r="E587" s="6" t="inlineStr"/>
       <c r="F587" s="7" t="n">
-        <v>84.01000000000001</v>
+        <v>61.69</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
@@ -25969,12 +25959,12 @@
       <c r="J587" s="6" t="inlineStr"/>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25982,35 +25972,29 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>79</v>
+        <v>6.16</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>-0.0271</v>
+        <v>0.0016</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>51500</v>
-      </c>
-      <c r="E588" s="4" t="n">
-        <v>0.58</v>
-      </c>
+        <v>7010000</v>
+      </c>
+      <c r="E588" s="2" t="inlineStr"/>
       <c r="F588" s="3" t="n">
-        <v>45.17</v>
+        <v>61.49</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="4" t="n">
-        <v>-9.409700000000001</v>
-      </c>
-      <c r="J588" s="4" t="n">
-        <v>-4.155</v>
-      </c>
+      <c r="I588" s="2" t="inlineStr"/>
+      <c r="J588" s="2" t="inlineStr"/>
       <c r="K588" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L588" s="2" t="inlineStr"/>
@@ -26019,40 +26003,34 @@
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>7.93</v>
+        <v>14.26</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0999</v>
+        <v>-0.0138</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>111200000</v>
-      </c>
-      <c r="E589" s="8" t="n">
-        <v>0.1672</v>
-      </c>
+        <v>30310000</v>
+      </c>
+      <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>65.98</v>
+        <v>56.21</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
-      <c r="I589" s="8" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J589" s="8" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I589" s="6" t="inlineStr"/>
+      <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L589" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M589" s="6" t="inlineStr"/>
@@ -26095,23 +26073,21 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>29.7</v>
+        <v>18.8</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0034</v>
+        <v>-0.0284</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>15250000</v>
-      </c>
-      <c r="E591" s="8" t="n">
-        <v>0.2667</v>
-      </c>
+        <v>81680000</v>
+      </c>
+      <c r="E591" s="6" t="inlineStr"/>
       <c r="F591" s="7" t="n">
-        <v>54.19</v>
+        <v>56.87</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
@@ -26119,12 +26095,12 @@
       <c r="J591" s="6" t="inlineStr"/>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L591" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M591" s="6" t="inlineStr"/>
@@ -26132,69 +26108,77 @@
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>195.3</v>
+        <v>79</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>0.0225</v>
+        <v>-0.0271</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>17690000</v>
-      </c>
-      <c r="E592" s="2" t="inlineStr"/>
+        <v>51500</v>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F592" s="3" t="n">
-        <v>48.2</v>
+        <v>45.17</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
-      <c r="I592" s="2" t="inlineStr"/>
-      <c r="J592" s="2" t="inlineStr"/>
+      <c r="I592" s="4" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J592" s="4" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr">
-        <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr"/>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>33.64</v>
+        <v>147</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>-0.01</v>
+        <v>0</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>3630000</v>
-      </c>
-      <c r="E593" s="6" t="inlineStr"/>
+        <v>1750000</v>
+      </c>
+      <c r="E593" s="8" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F593" s="7" t="n">
-        <v>51.56</v>
+        <v>50.74</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="6" t="inlineStr"/>
-      <c r="J593" s="6" t="inlineStr"/>
+      <c r="I593" s="8" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J593" s="8" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
+          <t>Perakende satış</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26202,23 +26186,23 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>240.6</v>
+        <v>29.7</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>0.0021</v>
+        <v>-0.0034</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>8440</v>
+        <v>15250000</v>
       </c>
       <c r="E594" s="4" t="n">
-        <v>0.2578</v>
+        <v>0.2667</v>
       </c>
       <c r="F594" s="3" t="n">
-        <v>41.2</v>
+        <v>54.19</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
@@ -26226,49 +26210,53 @@
       <c r="J594" s="2" t="inlineStr"/>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>147</v>
+        <v>2.7</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0</v>
+        <v>0.0266</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>1750000</v>
+        <v>33460000</v>
       </c>
       <c r="E595" s="8" t="n">
-        <v>0.1071</v>
+        <v>0.7119</v>
       </c>
       <c r="F595" s="7" t="n">
-        <v>50.74</v>
+        <v>44.09</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
       <c r="I595" s="8" t="n">
-        <v>-3.6635</v>
+        <v>-191.6342</v>
       </c>
       <c r="J595" s="8" t="n">
-        <v>-0.4897</v>
+        <v>-0.8093</v>
       </c>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26276,21 +26264,23 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>177.6</v>
+        <v>6.3</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>-0.005600000000000001</v>
+        <v>0.0379</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>6700000</v>
-      </c>
-      <c r="E596" s="2" t="inlineStr"/>
+        <v>51450000</v>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>0.8667</v>
+      </c>
       <c r="F596" s="3" t="n">
-        <v>62.01</v>
+        <v>84.01000000000001</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26298,12 +26288,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26311,77 +26301,75 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>18</v>
+        <v>240.6</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0375</v>
+        <v>0.0021</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>12330000</v>
+        <v>8440</v>
       </c>
       <c r="E597" s="8" t="n">
-        <v>0.9246</v>
+        <v>0.2578</v>
       </c>
       <c r="F597" s="7" t="n">
-        <v>58.4</v>
-      </c>
-      <c r="G597" s="7" t="n">
-        <v>170.13</v>
-      </c>
+        <v>41.2</v>
+      </c>
+      <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
-      <c r="I597" s="8" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J597" s="8" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I597" s="6" t="inlineStr"/>
+      <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr"/>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>28.8</v>
+        <v>18</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>-0.0144</v>
+        <v>0.0375</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>22500000</v>
-      </c>
-      <c r="E598" s="2" t="inlineStr"/>
+        <v>12330000</v>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F598" s="3" t="n">
-        <v>65.22</v>
-      </c>
-      <c r="G598" s="2" t="inlineStr"/>
+        <v>58.4</v>
+      </c>
+      <c r="G598" s="3" t="n">
+        <v>170.13</v>
+      </c>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="2" t="inlineStr"/>
-      <c r="J598" s="2" t="inlineStr"/>
+      <c r="I598" s="4" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J598" s="4" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L598" s="2" t="inlineStr">
         <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M598" s="2" t="inlineStr"/>
@@ -26389,38 +26377,34 @@
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>35.22</v>
+        <v>195.3</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.015</v>
+        <v>0.0225</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>6830000</v>
-      </c>
-      <c r="E599" s="8" t="n">
-        <v>0.3528</v>
-      </c>
+        <v>17690000</v>
+      </c>
+      <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>42.78</v>
+        <v>48.2</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
       <c r="I599" s="6" t="inlineStr"/>
-      <c r="J599" s="8" t="n">
-        <v>-1.4864</v>
-      </c>
+      <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26428,34 +26412,38 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>18.9</v>
+        <v>67.25</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>0.0289</v>
+        <v>-0.003</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>51420000</v>
-      </c>
-      <c r="E600" s="2" t="inlineStr"/>
+        <v>805670</v>
+      </c>
+      <c r="E600" s="4" t="n">
+        <v>0.3695000000000001</v>
+      </c>
       <c r="F600" s="3" t="n">
-        <v>31.39</v>
+        <v>61.15</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="2" t="inlineStr"/>
-      <c r="J600" s="2" t="inlineStr"/>
+      <c r="J600" s="4" t="n">
+        <v>0.4139</v>
+      </c>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26463,21 +26451,21 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>80.84999999999999</v>
+        <v>17.49</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0152</v>
-      </c>
-      <c r="D601" s="9" t="n">
-        <v>211300</v>
+        <v>-0.0224</v>
+      </c>
+      <c r="D601" s="7" t="n">
+        <v>66930000.00000001</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>10.34</v>
+        <v>54.24</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26488,181 +26476,169 @@
           <t>Finans</t>
         </is>
       </c>
-      <c r="L601" s="6" t="inlineStr"/>
+      <c r="L601" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M601" s="6" t="inlineStr"/>
     </row>
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>80.98999999999999</v>
+        <v>28.8</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>0.0152</v>
+        <v>-0.0144</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>9870000</v>
+        <v>22500000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>47.08</v>
+        <v>65.22</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
-      <c r="K602" s="2" t="inlineStr"/>
-      <c r="L602" s="2" t="inlineStr"/>
+      <c r="K602" s="2" t="inlineStr">
+        <is>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
+        </is>
+      </c>
+      <c r="L602" s="2" t="inlineStr">
+        <is>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
+        </is>
+      </c>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>7.42</v>
+        <v>2.85</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0993</v>
+        <v>0.0071</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>728700</v>
-      </c>
-      <c r="E603" s="8" t="n">
-        <v>0.95</v>
-      </c>
+        <v>200210000</v>
+      </c>
+      <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>44.55</v>
+        <v>52.25</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
-      <c r="I603" s="8" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J603" s="8" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L603" s="6" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L603" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M603" s="6" t="inlineStr"/>
     </row>
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>67.25</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.003</v>
+        <v>-0.0152</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>805670</v>
-      </c>
-      <c r="E604" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>211300</v>
+      </c>
+      <c r="E604" s="2" t="inlineStr"/>
       <c r="F604" s="3" t="n">
-        <v>61.15</v>
+        <v>10.34</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
       <c r="I604" s="2" t="inlineStr"/>
-      <c r="J604" s="4" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J604" s="2" t="inlineStr"/>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr"/>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>2.7</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0266</v>
+        <v>0.0152</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>33460000</v>
-      </c>
-      <c r="E605" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>9870000</v>
+      </c>
+      <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>44.09</v>
+        <v>47.08</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
-      <c r="I605" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J605" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
-      <c r="K605" s="6" t="inlineStr">
-        <is>
-          <t>Dağıtım servisleri</t>
-        </is>
-      </c>
-      <c r="L605" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
-        </is>
-      </c>
+      <c r="I605" s="6" t="inlineStr"/>
+      <c r="J605" s="6" t="inlineStr"/>
+      <c r="K605" s="6" t="inlineStr"/>
+      <c r="L605" s="6" t="inlineStr"/>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>18.29</v>
+        <v>7.93</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0135</v>
+        <v>-0.0999</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>847610</v>
+        <v>111200000</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.9869</v>
+        <v>0.1672</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>59.2</v>
+        <v>65.98</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
       <c r="I606" s="4" t="n">
-        <v>-0.2446</v>
+        <v>-5.3262</v>
       </c>
       <c r="J606" s="4" t="n">
-        <v>0.3246</v>
+        <v>-4.2562</v>
       </c>
       <c r="K606" s="2" t="inlineStr">
         <is>
@@ -26671,7 +26647,7 @@
       </c>
       <c r="L606" s="2" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M606" s="2" t="inlineStr"/>
@@ -26679,21 +26655,21 @@
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>14.26</v>
+        <v>177.6</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.0138</v>
+        <v>-0.005600000000000001</v>
       </c>
       <c r="D607" s="9" t="n">
-        <v>30310000</v>
+        <v>6700000</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>56.21</v>
+        <v>62.01</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26701,12 +26677,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26714,61 +26690,69 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>44</v>
+        <v>7.42</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0237</v>
+        <v>0.0993</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>13410000</v>
-      </c>
-      <c r="E608" s="2" t="inlineStr"/>
+        <v>728700</v>
+      </c>
+      <c r="E608" s="4" t="n">
+        <v>0.95</v>
+      </c>
       <c r="F608" s="3" t="n">
-        <v>61.69</v>
+        <v>44.55</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
-      <c r="I608" s="2" t="inlineStr"/>
-      <c r="J608" s="2" t="inlineStr"/>
+      <c r="I608" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J608" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
-        </is>
-      </c>
-      <c r="L608" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L608" s="2" t="inlineStr"/>
       <c r="M608" s="2" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>2.85</v>
+        <v>18.29</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>0.0071</v>
+        <v>-0.0135</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>200210000</v>
-      </c>
-      <c r="E609" s="6" t="inlineStr"/>
+        <v>847610</v>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>0.9869</v>
+      </c>
       <c r="F609" s="7" t="n">
-        <v>52.25</v>
+        <v>59.2</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
-      <c r="I609" s="6" t="inlineStr"/>
-      <c r="J609" s="6" t="inlineStr"/>
+      <c r="I609" s="8" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J609" s="8" t="n">
+        <v>0.3246</v>
+      </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
           <t>Finans</t>
@@ -26776,7 +26760,7 @@
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST MENKUL KIYM YO</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26784,21 +26768,21 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>18.8</v>
+        <v>18.9</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>-0.0284</v>
+        <v>0.0289</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>81680000</v>
+        <v>51420000</v>
       </c>
       <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>56.87</v>
+        <v>31.39</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26806,12 +26790,12 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26819,21 +26803,21 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>6.16</v>
+        <v>33.64</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>0.0016</v>
+        <v>-0.01</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>7010000</v>
+        <v>3630000</v>
       </c>
       <c r="E611" s="6" t="inlineStr"/>
       <c r="F611" s="7" t="n">
-        <v>61.49</v>
+        <v>51.56</v>
       </c>
       <c r="G611" s="6" t="inlineStr"/>
       <c r="H611" s="6" t="inlineStr"/>
@@ -26841,10 +26825,14 @@
       <c r="J611" s="6" t="inlineStr"/>
       <c r="K611" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L611" s="6" t="inlineStr"/>
+          <t>Üretici imalatı</t>
+        </is>
+      </c>
+      <c r="L611" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+        </is>
+      </c>
       <c r="M611" s="6" t="inlineStr"/>
     </row>
   </sheetData>
@@ -26869,7 +26857,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>06.05.2026 15:30</t>
+          <t>06.05.2026 16:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 BIST Screener | 06.05.2026 16:59 | 610 hisse
</commit_message>
<xml_diff>
--- a/data/bist_screener_2026-05-06.xlsx
+++ b/data/bist_screener_2026-05-06.xlsx
@@ -25898,38 +25898,38 @@
     <row r="586">
       <c r="A586" s="2" t="inlineStr">
         <is>
-          <t>LILAK</t>
+          <t>NETAS</t>
         </is>
       </c>
       <c r="B586" s="3" t="n">
-        <v>35.22</v>
+        <v>67.25</v>
       </c>
       <c r="C586" s="4" t="n">
-        <v>0.015</v>
+        <v>-0.003</v>
       </c>
       <c r="D586" s="5" t="n">
-        <v>6830000</v>
+        <v>805670</v>
       </c>
       <c r="E586" s="4" t="n">
-        <v>0.3528</v>
+        <v>0.3695000000000001</v>
       </c>
       <c r="F586" s="3" t="n">
-        <v>42.78</v>
+        <v>61.15</v>
       </c>
       <c r="G586" s="2" t="inlineStr"/>
       <c r="H586" s="2" t="inlineStr"/>
       <c r="I586" s="2" t="inlineStr"/>
       <c r="J586" s="4" t="n">
-        <v>-1.4864</v>
+        <v>0.4139</v>
       </c>
       <c r="K586" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı olmayan tüketici ürünleri</t>
+          <t>Teknoloji hizmetleri</t>
         </is>
       </c>
       <c r="L586" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M586" s="2" t="inlineStr"/>
@@ -25937,34 +25937,38 @@
     <row r="587">
       <c r="A587" s="6" t="inlineStr">
         <is>
-          <t>EMPAE</t>
+          <t>LILAK</t>
         </is>
       </c>
       <c r="B587" s="7" t="n">
-        <v>44</v>
+        <v>35.22</v>
       </c>
       <c r="C587" s="8" t="n">
-        <v>0.0237</v>
+        <v>0.015</v>
       </c>
       <c r="D587" s="9" t="n">
-        <v>13410000</v>
-      </c>
-      <c r="E587" s="6" t="inlineStr"/>
+        <v>6830000</v>
+      </c>
+      <c r="E587" s="8" t="n">
+        <v>0.3528</v>
+      </c>
       <c r="F587" s="7" t="n">
-        <v>61.69</v>
+        <v>42.78</v>
       </c>
       <c r="G587" s="6" t="inlineStr"/>
       <c r="H587" s="6" t="inlineStr"/>
       <c r="I587" s="6" t="inlineStr"/>
-      <c r="J587" s="6" t="inlineStr"/>
+      <c r="J587" s="8" t="n">
+        <v>-1.4864</v>
+      </c>
       <c r="K587" s="6" t="inlineStr">
         <is>
-          <t>Elektronik teknoloji</t>
+          <t>Dayanıklı olmayan tüketici ürünleri</t>
         </is>
       </c>
       <c r="L587" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST HALKA ARZ, BIST ORMAN KAĞIT BASIM, BIST YILDIZ, BIST TEMETTU, BIST KURUMSAL YÖNETİM, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M587" s="6" t="inlineStr"/>
@@ -25972,52 +25976,62 @@
     <row r="588">
       <c r="A588" s="2" t="inlineStr">
         <is>
-          <t>DMLKT</t>
+          <t>GRNYO</t>
         </is>
       </c>
       <c r="B588" s="3" t="n">
-        <v>6.16</v>
+        <v>18.29</v>
       </c>
       <c r="C588" s="4" t="n">
-        <v>0.0016</v>
+        <v>-0.0135</v>
       </c>
       <c r="D588" s="5" t="n">
-        <v>7010000</v>
-      </c>
-      <c r="E588" s="2" t="inlineStr"/>
+        <v>847610</v>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>0.9869</v>
+      </c>
       <c r="F588" s="3" t="n">
-        <v>61.49</v>
+        <v>59.2</v>
       </c>
       <c r="G588" s="2" t="inlineStr"/>
       <c r="H588" s="2" t="inlineStr"/>
-      <c r="I588" s="2" t="inlineStr"/>
-      <c r="J588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="n">
+        <v>-0.2446</v>
+      </c>
+      <c r="J588" s="4" t="n">
+        <v>0.3246</v>
+      </c>
       <c r="K588" s="2" t="inlineStr">
         <is>
           <t>Finans</t>
         </is>
       </c>
-      <c r="L588" s="2" t="inlineStr"/>
+      <c r="L588" s="2" t="inlineStr">
+        <is>
+          <t>BIST MENKUL KIYM YO</t>
+        </is>
+      </c>
       <c r="M588" s="2" t="inlineStr"/>
     </row>
     <row r="589">
       <c r="A589" s="6" t="inlineStr">
         <is>
-          <t>GENKM</t>
+          <t>ENPRA</t>
         </is>
       </c>
       <c r="B589" s="7" t="n">
-        <v>14.26</v>
+        <v>80.84999999999999</v>
       </c>
       <c r="C589" s="8" t="n">
-        <v>-0.0138</v>
+        <v>-0.0152</v>
       </c>
       <c r="D589" s="9" t="n">
-        <v>30310000</v>
+        <v>211300</v>
       </c>
       <c r="E589" s="6" t="inlineStr"/>
       <c r="F589" s="7" t="n">
-        <v>56.21</v>
+        <v>10.34</v>
       </c>
       <c r="G589" s="6" t="inlineStr"/>
       <c r="H589" s="6" t="inlineStr"/>
@@ -26025,34 +26039,30 @@
       <c r="J589" s="6" t="inlineStr"/>
       <c r="K589" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L589" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L589" s="6" t="inlineStr"/>
       <c r="M589" s="6" t="inlineStr"/>
     </row>
     <row r="590">
       <c r="A590" s="2" t="inlineStr">
         <is>
-          <t>CGCAM</t>
+          <t>AAGYO</t>
         </is>
       </c>
       <c r="B590" s="3" t="n">
-        <v>42.6</v>
+        <v>18.9</v>
       </c>
       <c r="C590" s="4" t="n">
-        <v>0.0109</v>
+        <v>0.0289</v>
       </c>
       <c r="D590" s="5" t="n">
-        <v>5970000</v>
+        <v>51420000</v>
       </c>
       <c r="E590" s="2" t="inlineStr"/>
       <c r="F590" s="3" t="n">
-        <v>60.43</v>
+        <v>31.39</v>
       </c>
       <c r="G590" s="2" t="inlineStr"/>
       <c r="H590" s="2" t="inlineStr"/>
@@ -26060,12 +26070,12 @@
       <c r="J590" s="2" t="inlineStr"/>
       <c r="K590" s="2" t="inlineStr">
         <is>
-          <t>Dayanıklı tüketim malları</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L590" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
         </is>
       </c>
       <c r="M590" s="2" t="inlineStr"/>
@@ -26073,112 +26083,114 @@
     <row r="591">
       <c r="A591" s="6" t="inlineStr">
         <is>
-          <t>SMRVA</t>
+          <t>MMCAS</t>
         </is>
       </c>
       <c r="B591" s="7" t="n">
-        <v>18.8</v>
+        <v>79</v>
       </c>
       <c r="C591" s="8" t="n">
-        <v>-0.0284</v>
+        <v>-0.0271</v>
       </c>
       <c r="D591" s="9" t="n">
-        <v>81680000</v>
-      </c>
-      <c r="E591" s="6" t="inlineStr"/>
+        <v>51500</v>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>0.58</v>
+      </c>
       <c r="F591" s="7" t="n">
-        <v>56.87</v>
+        <v>45.17</v>
       </c>
       <c r="G591" s="6" t="inlineStr"/>
       <c r="H591" s="6" t="inlineStr"/>
-      <c r="I591" s="6" t="inlineStr"/>
-      <c r="J591" s="6" t="inlineStr"/>
+      <c r="I591" s="8" t="n">
+        <v>-9.409700000000001</v>
+      </c>
+      <c r="J591" s="8" t="n">
+        <v>-4.155</v>
+      </c>
       <c r="K591" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
-        </is>
-      </c>
-      <c r="L591" s="6" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
-        </is>
-      </c>
+          <t>Taşımacılık</t>
+        </is>
+      </c>
+      <c r="L591" s="6" t="inlineStr"/>
       <c r="M591" s="6" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" s="2" t="inlineStr">
         <is>
-          <t>MMCAS</t>
+          <t>BORLS</t>
         </is>
       </c>
       <c r="B592" s="3" t="n">
-        <v>79</v>
+        <v>7.93</v>
       </c>
       <c r="C592" s="4" t="n">
-        <v>-0.0271</v>
+        <v>-0.0999</v>
       </c>
       <c r="D592" s="5" t="n">
-        <v>51500</v>
+        <v>111200000</v>
       </c>
       <c r="E592" s="4" t="n">
-        <v>0.58</v>
+        <v>0.1672</v>
       </c>
       <c r="F592" s="3" t="n">
-        <v>45.17</v>
+        <v>65.98</v>
       </c>
       <c r="G592" s="2" t="inlineStr"/>
       <c r="H592" s="2" t="inlineStr"/>
       <c r="I592" s="4" t="n">
-        <v>-9.409700000000001</v>
+        <v>-5.3262</v>
       </c>
       <c r="J592" s="4" t="n">
-        <v>-4.155</v>
+        <v>-4.2562</v>
       </c>
       <c r="K592" s="2" t="inlineStr">
         <is>
-          <t>Taşımacılık</t>
-        </is>
-      </c>
-      <c r="L592" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L592" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
+        </is>
+      </c>
       <c r="M592" s="2" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" s="6" t="inlineStr">
         <is>
-          <t>CRFSA</t>
+          <t>UCAYM</t>
         </is>
       </c>
       <c r="B593" s="7" t="n">
-        <v>147</v>
+        <v>29.7</v>
       </c>
       <c r="C593" s="8" t="n">
-        <v>0</v>
+        <v>-0.0034</v>
       </c>
       <c r="D593" s="9" t="n">
-        <v>1750000</v>
+        <v>15250000</v>
       </c>
       <c r="E593" s="8" t="n">
-        <v>0.1071</v>
+        <v>0.2667</v>
       </c>
       <c r="F593" s="7" t="n">
-        <v>50.74</v>
+        <v>54.19</v>
       </c>
       <c r="G593" s="6" t="inlineStr"/>
       <c r="H593" s="6" t="inlineStr"/>
-      <c r="I593" s="8" t="n">
-        <v>-3.6635</v>
-      </c>
-      <c r="J593" s="8" t="n">
-        <v>-0.4897</v>
-      </c>
+      <c r="I593" s="6" t="inlineStr"/>
+      <c r="J593" s="6" t="inlineStr"/>
       <c r="K593" s="6" t="inlineStr">
         <is>
-          <t>Perakende satış</t>
+          <t>Endüstriyel hizmetler</t>
         </is>
       </c>
       <c r="L593" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M593" s="6" t="inlineStr"/>
@@ -26186,77 +26198,71 @@
     <row r="594">
       <c r="A594" s="2" t="inlineStr">
         <is>
-          <t>UCAYM</t>
+          <t>BRMEN</t>
         </is>
       </c>
       <c r="B594" s="3" t="n">
-        <v>29.7</v>
+        <v>7.42</v>
       </c>
       <c r="C594" s="4" t="n">
-        <v>-0.0034</v>
+        <v>0.0993</v>
       </c>
       <c r="D594" s="5" t="n">
-        <v>15250000</v>
+        <v>728700</v>
       </c>
       <c r="E594" s="4" t="n">
-        <v>0.2667</v>
+        <v>0.95</v>
       </c>
       <c r="F594" s="3" t="n">
-        <v>54.19</v>
+        <v>44.55</v>
       </c>
       <c r="G594" s="2" t="inlineStr"/>
       <c r="H594" s="2" t="inlineStr"/>
-      <c r="I594" s="2" t="inlineStr"/>
-      <c r="J594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="n">
+        <v>-23.6291</v>
+      </c>
+      <c r="J594" s="4" t="n">
+        <v>-0.4678</v>
+      </c>
       <c r="K594" s="2" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
-        </is>
-      </c>
-      <c r="L594" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L594" s="2" t="inlineStr"/>
       <c r="M594" s="2" t="inlineStr"/>
     </row>
     <row r="595">
       <c r="A595" s="6" t="inlineStr">
         <is>
-          <t>ARZUM</t>
+          <t>MCARD</t>
         </is>
       </c>
       <c r="B595" s="7" t="n">
-        <v>2.7</v>
+        <v>177.6</v>
       </c>
       <c r="C595" s="8" t="n">
-        <v>0.0266</v>
+        <v>-0.005600000000000001</v>
       </c>
       <c r="D595" s="9" t="n">
-        <v>33460000</v>
-      </c>
-      <c r="E595" s="8" t="n">
-        <v>0.7119</v>
-      </c>
+        <v>6700000</v>
+      </c>
+      <c r="E595" s="6" t="inlineStr"/>
       <c r="F595" s="7" t="n">
-        <v>44.09</v>
+        <v>62.01</v>
       </c>
       <c r="G595" s="6" t="inlineStr"/>
       <c r="H595" s="6" t="inlineStr"/>
-      <c r="I595" s="8" t="n">
-        <v>-191.6342</v>
-      </c>
-      <c r="J595" s="8" t="n">
-        <v>-0.8093</v>
-      </c>
+      <c r="I595" s="6" t="inlineStr"/>
+      <c r="J595" s="6" t="inlineStr"/>
       <c r="K595" s="6" t="inlineStr">
         <is>
-          <t>Dağıtım servisleri</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L595" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M595" s="6" t="inlineStr"/>
@@ -26264,23 +26270,21 @@
     <row r="596">
       <c r="A596" s="2" t="inlineStr">
         <is>
-          <t>ICUGS</t>
+          <t>CGCAM</t>
         </is>
       </c>
       <c r="B596" s="3" t="n">
-        <v>6.3</v>
+        <v>42.6</v>
       </c>
       <c r="C596" s="4" t="n">
-        <v>0.0379</v>
+        <v>0.0109</v>
       </c>
       <c r="D596" s="5" t="n">
-        <v>51450000</v>
-      </c>
-      <c r="E596" s="4" t="n">
-        <v>0.8667</v>
-      </c>
+        <v>5970000</v>
+      </c>
+      <c r="E596" s="2" t="inlineStr"/>
       <c r="F596" s="3" t="n">
-        <v>84.01000000000001</v>
+        <v>60.43</v>
       </c>
       <c r="G596" s="2" t="inlineStr"/>
       <c r="H596" s="2" t="inlineStr"/>
@@ -26288,12 +26292,12 @@
       <c r="J596" s="2" t="inlineStr"/>
       <c r="K596" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dayanıklı tüketim malları</t>
         </is>
       </c>
       <c r="L596" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST TAŞ TOPRAK, BIST HALKA ARZ, BIST ANA, BIST MANİSA</t>
         </is>
       </c>
       <c r="M596" s="2" t="inlineStr"/>
@@ -26301,23 +26305,21 @@
     <row r="597">
       <c r="A597" s="6" t="inlineStr">
         <is>
-          <t>INTEK</t>
+          <t>GLRMK</t>
         </is>
       </c>
       <c r="B597" s="7" t="n">
-        <v>240.6</v>
+        <v>195.3</v>
       </c>
       <c r="C597" s="8" t="n">
-        <v>0.0021</v>
+        <v>0.0225</v>
       </c>
       <c r="D597" s="9" t="n">
-        <v>8440</v>
-      </c>
-      <c r="E597" s="8" t="n">
-        <v>0.2578</v>
-      </c>
+        <v>17690000</v>
+      </c>
+      <c r="E597" s="6" t="inlineStr"/>
       <c r="F597" s="7" t="n">
-        <v>41.2</v>
+        <v>48.2</v>
       </c>
       <c r="G597" s="6" t="inlineStr"/>
       <c r="H597" s="6" t="inlineStr"/>
@@ -26325,73 +26327,65 @@
       <c r="J597" s="6" t="inlineStr"/>
       <c r="K597" s="6" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L597" s="6" t="inlineStr"/>
+          <t>Endüstriyel hizmetler</t>
+        </is>
+      </c>
+      <c r="L597" s="6" t="inlineStr">
+        <is>
+          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+        </is>
+      </c>
       <c r="M597" s="6" t="inlineStr"/>
     </row>
     <row r="598">
       <c r="A598" s="2" t="inlineStr">
         <is>
-          <t>BERA</t>
+          <t>DMLKT</t>
         </is>
       </c>
       <c r="B598" s="3" t="n">
-        <v>18</v>
+        <v>6.16</v>
       </c>
       <c r="C598" s="4" t="n">
-        <v>0.0375</v>
+        <v>0.0016</v>
       </c>
       <c r="D598" s="5" t="n">
-        <v>12330000</v>
-      </c>
-      <c r="E598" s="4" t="n">
-        <v>0.9246</v>
-      </c>
+        <v>7010000</v>
+      </c>
+      <c r="E598" s="2" t="inlineStr"/>
       <c r="F598" s="3" t="n">
-        <v>58.4</v>
-      </c>
-      <c r="G598" s="3" t="n">
-        <v>170.13</v>
-      </c>
+        <v>61.49</v>
+      </c>
+      <c r="G598" s="2" t="inlineStr"/>
       <c r="H598" s="2" t="inlineStr"/>
-      <c r="I598" s="4" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="J598" s="4" t="n">
-        <v>-10.3171</v>
-      </c>
+      <c r="I598" s="2" t="inlineStr"/>
+      <c r="J598" s="2" t="inlineStr"/>
       <c r="K598" s="2" t="inlineStr">
         <is>
-          <t>Üretici imalatı</t>
-        </is>
-      </c>
-      <c r="L598" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
-        </is>
-      </c>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L598" s="2" t="inlineStr"/>
       <c r="M598" s="2" t="inlineStr"/>
     </row>
     <row r="599">
       <c r="A599" s="6" t="inlineStr">
         <is>
-          <t>GLRMK</t>
+          <t>BESTE</t>
         </is>
       </c>
       <c r="B599" s="7" t="n">
-        <v>195.3</v>
+        <v>28.8</v>
       </c>
       <c r="C599" s="8" t="n">
-        <v>0.0225</v>
+        <v>-0.0144</v>
       </c>
       <c r="D599" s="9" t="n">
-        <v>17690000</v>
+        <v>22500000</v>
       </c>
       <c r="E599" s="6" t="inlineStr"/>
       <c r="F599" s="7" t="n">
-        <v>48.2</v>
+        <v>65.22</v>
       </c>
       <c r="G599" s="6" t="inlineStr"/>
       <c r="H599" s="6" t="inlineStr"/>
@@ -26399,12 +26393,12 @@
       <c r="J599" s="6" t="inlineStr"/>
       <c r="K599" s="6" t="inlineStr">
         <is>
-          <t>Endüstriyel hizmetler</t>
+          <t>Elektrik, Su, Gaz Hizmetleri</t>
         </is>
       </c>
       <c r="L599" s="6" t="inlineStr">
         <is>
-          <t>BIST 100, BIST 100 AĞIRLIK SINIRLAMALI 10, BIST TÜM, BIST İNŞAAT, BIST HALKA ARZ, BIST HİZMETLER, BIST 100-30, BIST KATILIM 100, BIST KATILIM TÜM, BIST 100 AĞIRLIK SINIRLAMALI 25, BIST YILDIZ, BIST KATILIM 50, BIST KATILIM 30, BIST ANKARA, BIST KATILIM 30 EŞİT AĞIRLIKLI GETİRİ</t>
+          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M599" s="6" t="inlineStr"/>
@@ -26412,38 +26406,34 @@
     <row r="600">
       <c r="A600" s="2" t="inlineStr">
         <is>
-          <t>NETAS</t>
+          <t>FRMPL</t>
         </is>
       </c>
       <c r="B600" s="3" t="n">
-        <v>67.25</v>
+        <v>33.64</v>
       </c>
       <c r="C600" s="4" t="n">
-        <v>-0.003</v>
+        <v>-0.01</v>
       </c>
       <c r="D600" s="5" t="n">
-        <v>805670</v>
-      </c>
-      <c r="E600" s="4" t="n">
-        <v>0.3695000000000001</v>
-      </c>
+        <v>3630000</v>
+      </c>
+      <c r="E600" s="2" t="inlineStr"/>
       <c r="F600" s="3" t="n">
-        <v>61.15</v>
+        <v>51.56</v>
       </c>
       <c r="G600" s="2" t="inlineStr"/>
       <c r="H600" s="2" t="inlineStr"/>
       <c r="I600" s="2" t="inlineStr"/>
-      <c r="J600" s="4" t="n">
-        <v>0.4139</v>
-      </c>
+      <c r="J600" s="2" t="inlineStr"/>
       <c r="K600" s="2" t="inlineStr">
         <is>
-          <t>Teknoloji hizmetleri</t>
+          <t>Üretici imalatı</t>
         </is>
       </c>
       <c r="L600" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KURUMSAL YÖNETİM</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
         </is>
       </c>
       <c r="M600" s="2" t="inlineStr"/>
@@ -26451,21 +26441,21 @@
     <row r="601">
       <c r="A601" s="6" t="inlineStr">
         <is>
-          <t>LXGYO</t>
+          <t>EMPAE</t>
         </is>
       </c>
       <c r="B601" s="7" t="n">
-        <v>17.49</v>
+        <v>44</v>
       </c>
       <c r="C601" s="8" t="n">
-        <v>-0.0224</v>
-      </c>
-      <c r="D601" s="7" t="n">
-        <v>66930000.00000001</v>
+        <v>0.0237</v>
+      </c>
+      <c r="D601" s="9" t="n">
+        <v>13410000</v>
       </c>
       <c r="E601" s="6" t="inlineStr"/>
       <c r="F601" s="7" t="n">
-        <v>54.24</v>
+        <v>61.69</v>
       </c>
       <c r="G601" s="6" t="inlineStr"/>
       <c r="H601" s="6" t="inlineStr"/>
@@ -26473,12 +26463,12 @@
       <c r="J601" s="6" t="inlineStr"/>
       <c r="K601" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Elektronik teknoloji</t>
         </is>
       </c>
       <c r="L601" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
         </is>
       </c>
       <c r="M601" s="6" t="inlineStr"/>
@@ -26486,56 +26476,48 @@
     <row r="602">
       <c r="A602" s="2" t="inlineStr">
         <is>
-          <t>BESTE</t>
+          <t>ALTIN</t>
         </is>
       </c>
       <c r="B602" s="3" t="n">
-        <v>28.8</v>
+        <v>80.98999999999999</v>
       </c>
       <c r="C602" s="4" t="n">
-        <v>-0.0144</v>
+        <v>0.0152</v>
       </c>
       <c r="D602" s="5" t="n">
-        <v>22500000</v>
+        <v>9870000</v>
       </c>
       <c r="E602" s="2" t="inlineStr"/>
       <c r="F602" s="3" t="n">
-        <v>65.22</v>
+        <v>47.08</v>
       </c>
       <c r="G602" s="2" t="inlineStr"/>
       <c r="H602" s="2" t="inlineStr"/>
       <c r="I602" s="2" t="inlineStr"/>
       <c r="J602" s="2" t="inlineStr"/>
-      <c r="K602" s="2" t="inlineStr">
-        <is>
-          <t>Elektrik, Su, Gaz Hizmetleri</t>
-        </is>
-      </c>
-      <c r="L602" s="2" t="inlineStr">
-        <is>
-          <t>BIST ELEKTRIK, BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST HİZMETLER, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA</t>
-        </is>
-      </c>
+      <c r="K602" s="2" t="inlineStr"/>
+      <c r="L602" s="2" t="inlineStr"/>
       <c r="M602" s="2" t="inlineStr"/>
     </row>
     <row r="603">
       <c r="A603" s="6" t="inlineStr">
         <is>
-          <t>MARMR</t>
+          <t>GENKM</t>
         </is>
       </c>
       <c r="B603" s="7" t="n">
-        <v>2.85</v>
+        <v>14.26</v>
       </c>
       <c r="C603" s="8" t="n">
-        <v>0.0071</v>
+        <v>-0.0138</v>
       </c>
       <c r="D603" s="9" t="n">
-        <v>200210000</v>
+        <v>30310000</v>
       </c>
       <c r="E603" s="6" t="inlineStr"/>
       <c r="F603" s="7" t="n">
-        <v>52.25</v>
+        <v>56.21</v>
       </c>
       <c r="G603" s="6" t="inlineStr"/>
       <c r="H603" s="6" t="inlineStr"/>
@@ -26543,12 +26525,12 @@
       <c r="J603" s="6" t="inlineStr"/>
       <c r="K603" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>İşlenebilen endüstriler</t>
         </is>
       </c>
       <c r="L603" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST KOCAELI</t>
         </is>
       </c>
       <c r="M603" s="6" t="inlineStr"/>
@@ -26556,120 +26538,130 @@
     <row r="604">
       <c r="A604" s="2" t="inlineStr">
         <is>
-          <t>ENPRA</t>
+          <t>CRFSA</t>
         </is>
       </c>
       <c r="B604" s="3" t="n">
-        <v>80.84999999999999</v>
+        <v>147</v>
       </c>
       <c r="C604" s="4" t="n">
-        <v>-0.0152</v>
+        <v>0</v>
       </c>
       <c r="D604" s="5" t="n">
-        <v>211300</v>
-      </c>
-      <c r="E604" s="2" t="inlineStr"/>
+        <v>1750000</v>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>0.1071</v>
+      </c>
       <c r="F604" s="3" t="n">
-        <v>10.34</v>
+        <v>50.74</v>
       </c>
       <c r="G604" s="2" t="inlineStr"/>
       <c r="H604" s="2" t="inlineStr"/>
-      <c r="I604" s="2" t="inlineStr"/>
-      <c r="J604" s="2" t="inlineStr"/>
+      <c r="I604" s="4" t="n">
+        <v>-3.6635</v>
+      </c>
+      <c r="J604" s="4" t="n">
+        <v>-0.4897</v>
+      </c>
       <c r="K604" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L604" s="2" t="inlineStr"/>
+          <t>Perakende satış</t>
+        </is>
+      </c>
+      <c r="L604" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST ANA</t>
+        </is>
+      </c>
       <c r="M604" s="2" t="inlineStr"/>
     </row>
     <row r="605">
       <c r="A605" s="6" t="inlineStr">
         <is>
-          <t>ALTIN</t>
+          <t>MARMR</t>
         </is>
       </c>
       <c r="B605" s="7" t="n">
-        <v>80.98999999999999</v>
+        <v>2.85</v>
       </c>
       <c r="C605" s="8" t="n">
-        <v>0.0152</v>
+        <v>0.0071</v>
       </c>
       <c r="D605" s="9" t="n">
-        <v>9870000</v>
+        <v>200210000</v>
       </c>
       <c r="E605" s="6" t="inlineStr"/>
       <c r="F605" s="7" t="n">
-        <v>47.08</v>
+        <v>52.25</v>
       </c>
       <c r="G605" s="6" t="inlineStr"/>
       <c r="H605" s="6" t="inlineStr"/>
       <c r="I605" s="6" t="inlineStr"/>
       <c r="J605" s="6" t="inlineStr"/>
-      <c r="K605" s="6" t="inlineStr"/>
-      <c r="L605" s="6" t="inlineStr"/>
+      <c r="K605" s="6" t="inlineStr">
+        <is>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L605" s="6" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST ANA, BIST KOCAELI</t>
+        </is>
+      </c>
       <c r="M605" s="6" t="inlineStr"/>
     </row>
     <row r="606">
       <c r="A606" s="2" t="inlineStr">
         <is>
-          <t>BORLS</t>
+          <t>INTEK</t>
         </is>
       </c>
       <c r="B606" s="3" t="n">
-        <v>7.93</v>
+        <v>240.6</v>
       </c>
       <c r="C606" s="4" t="n">
-        <v>-0.0999</v>
+        <v>0.0021</v>
       </c>
       <c r="D606" s="5" t="n">
-        <v>111200000</v>
+        <v>8440</v>
       </c>
       <c r="E606" s="4" t="n">
-        <v>0.1672</v>
+        <v>0.2578</v>
       </c>
       <c r="F606" s="3" t="n">
-        <v>65.98</v>
+        <v>41.2</v>
       </c>
       <c r="G606" s="2" t="inlineStr"/>
       <c r="H606" s="2" t="inlineStr"/>
-      <c r="I606" s="4" t="n">
-        <v>-5.3262</v>
-      </c>
-      <c r="J606" s="4" t="n">
-        <v>-4.2562</v>
-      </c>
+      <c r="I606" s="2" t="inlineStr"/>
+      <c r="J606" s="2" t="inlineStr"/>
       <c r="K606" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
-        </is>
-      </c>
-      <c r="L606" s="2" t="inlineStr">
-        <is>
-          <t>BIST TUM-100, BIST TÜM, BIST HİZMETLER, BIST İSTANBUL, BIST YILDIZ</t>
-        </is>
-      </c>
+          <t>İşlenebilen endüstriler</t>
+        </is>
+      </c>
+      <c r="L606" s="2" t="inlineStr"/>
       <c r="M606" s="2" t="inlineStr"/>
     </row>
     <row r="607">
       <c r="A607" s="6" t="inlineStr">
         <is>
-          <t>MCARD</t>
+          <t>LXGYO</t>
         </is>
       </c>
       <c r="B607" s="7" t="n">
-        <v>177.6</v>
+        <v>17.49</v>
       </c>
       <c r="C607" s="8" t="n">
-        <v>-0.005600000000000001</v>
-      </c>
-      <c r="D607" s="9" t="n">
-        <v>6700000</v>
+        <v>-0.0224</v>
+      </c>
+      <c r="D607" s="7" t="n">
+        <v>66930000.00000001</v>
       </c>
       <c r="E607" s="6" t="inlineStr"/>
       <c r="F607" s="7" t="n">
-        <v>62.01</v>
+        <v>54.24</v>
       </c>
       <c r="G607" s="6" t="inlineStr"/>
       <c r="H607" s="6" t="inlineStr"/>
@@ -26677,12 +26669,12 @@
       <c r="J607" s="6" t="inlineStr"/>
       <c r="K607" s="6" t="inlineStr">
         <is>
-          <t>Ticari hizmetler</t>
+          <t>Finans</t>
         </is>
       </c>
       <c r="L607" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST TEKNOLOJİ, BIST BILISIM, BIST HALKA ARZ, BIST İSTANBUL, BIST KATILIM TÜM, BIST ANA, BIST TEMETTU, BIST TEKNOLOJI AĞIRLIK SINIRLAMALI, BIST KATILIM TEMETTU</t>
+          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST ANA</t>
         </is>
       </c>
       <c r="M607" s="6" t="inlineStr"/>
@@ -26690,77 +26682,77 @@
     <row r="608">
       <c r="A608" s="2" t="inlineStr">
         <is>
-          <t>BRMEN</t>
+          <t>ICUGS</t>
         </is>
       </c>
       <c r="B608" s="3" t="n">
-        <v>7.42</v>
+        <v>6.3</v>
       </c>
       <c r="C608" s="4" t="n">
-        <v>0.0993</v>
+        <v>0.0379</v>
       </c>
       <c r="D608" s="5" t="n">
-        <v>728700</v>
+        <v>51450000</v>
       </c>
       <c r="E608" s="4" t="n">
-        <v>0.95</v>
+        <v>0.8667</v>
       </c>
       <c r="F608" s="3" t="n">
-        <v>44.55</v>
+        <v>84.01000000000001</v>
       </c>
       <c r="G608" s="2" t="inlineStr"/>
       <c r="H608" s="2" t="inlineStr"/>
-      <c r="I608" s="4" t="n">
-        <v>-23.6291</v>
-      </c>
-      <c r="J608" s="4" t="n">
-        <v>-0.4678</v>
-      </c>
+      <c r="I608" s="2" t="inlineStr"/>
+      <c r="J608" s="2" t="inlineStr"/>
       <c r="K608" s="2" t="inlineStr">
         <is>
-          <t>İşlenebilen endüstriler</t>
-        </is>
-      </c>
-      <c r="L608" s="2" t="inlineStr"/>
+          <t>Finans</t>
+        </is>
+      </c>
+      <c r="L608" s="2" t="inlineStr">
+        <is>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST ANA</t>
+        </is>
+      </c>
       <c r="M608" s="2" t="inlineStr"/>
     </row>
     <row r="609">
       <c r="A609" s="6" t="inlineStr">
         <is>
-          <t>GRNYO</t>
+          <t>ARZUM</t>
         </is>
       </c>
       <c r="B609" s="7" t="n">
-        <v>18.29</v>
+        <v>2.7</v>
       </c>
       <c r="C609" s="8" t="n">
-        <v>-0.0135</v>
+        <v>0.0266</v>
       </c>
       <c r="D609" s="9" t="n">
-        <v>847610</v>
+        <v>33460000</v>
       </c>
       <c r="E609" s="8" t="n">
-        <v>0.9869</v>
+        <v>0.7119</v>
       </c>
       <c r="F609" s="7" t="n">
-        <v>59.2</v>
+        <v>44.09</v>
       </c>
       <c r="G609" s="6" t="inlineStr"/>
       <c r="H609" s="6" t="inlineStr"/>
       <c r="I609" s="8" t="n">
-        <v>-0.2446</v>
+        <v>-191.6342</v>
       </c>
       <c r="J609" s="8" t="n">
-        <v>0.3246</v>
+        <v>-0.8093</v>
       </c>
       <c r="K609" s="6" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Dağıtım servisleri</t>
         </is>
       </c>
       <c r="L609" s="6" t="inlineStr">
         <is>
-          <t>BIST MENKUL KIYM YO</t>
+          <t>BIST TUM-100, BIST TÜM, BIST TİCARET, BIST HİZMETLER, BIST İSTANBUL, BIST ANA, BIST KURUMSAL YÖNETİM</t>
         </is>
       </c>
       <c r="M609" s="6" t="inlineStr"/>
@@ -26768,21 +26760,21 @@
     <row r="610">
       <c r="A610" s="2" t="inlineStr">
         <is>
-          <t>AAGYO</t>
+          <t>SMRVA</t>
         </is>
       </c>
       <c r="B610" s="3" t="n">
-        <v>18.9</v>
+        <v>18.8</v>
       </c>
       <c r="C610" s="4" t="n">
-        <v>0.0289</v>
+        <v>-0.0284</v>
       </c>
       <c r="D610" s="5" t="n">
-        <v>51420000</v>
+        <v>81680000</v>
       </c>
       <c r="E610" s="2" t="inlineStr"/>
       <c r="F610" s="3" t="n">
-        <v>31.39</v>
+        <v>56.87</v>
       </c>
       <c r="G610" s="2" t="inlineStr"/>
       <c r="H610" s="2" t="inlineStr"/>
@@ -26790,12 +26782,12 @@
       <c r="J610" s="2" t="inlineStr"/>
       <c r="K610" s="2" t="inlineStr">
         <is>
-          <t>Finans</t>
+          <t>Ticari hizmetler</t>
         </is>
       </c>
       <c r="L610" s="2" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST TÜM, BIST GAYRİMENKUL YO, BIST HALKA ARZ, BIST MALİ, BIST KATILIM TÜM, BIST YILDIZ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HALKA ARZ, BIST MALİ, BIST ANA, BIST TEMETTU</t>
         </is>
       </c>
       <c r="M610" s="2" t="inlineStr"/>
@@ -26803,26 +26795,34 @@
     <row r="611">
       <c r="A611" s="6" t="inlineStr">
         <is>
-          <t>FRMPL</t>
+          <t>BERA</t>
         </is>
       </c>
       <c r="B611" s="7" t="n">
-        <v>33.64</v>
+        <v>18</v>
       </c>
       <c r="C611" s="8" t="n">
-        <v>-0.01</v>
+        <v>0.0375</v>
       </c>
       <c r="D611" s="9" t="n">
-        <v>3630000</v>
-      </c>
-      <c r="E611" s="6" t="inlineStr"/>
+        <v>12330000</v>
+      </c>
+      <c r="E611" s="8" t="n">
+        <v>0.9246</v>
+      </c>
       <c r="F611" s="7" t="n">
-        <v>51.56</v>
-      </c>
-      <c r="G611" s="6" t="inlineStr"/>
+        <v>58.4</v>
+      </c>
+      <c r="G611" s="7" t="n">
+        <v>170.13</v>
+      </c>
       <c r="H611" s="6" t="inlineStr"/>
-      <c r="I611" s="6" t="inlineStr"/>
-      <c r="J611" s="6" t="inlineStr"/>
+      <c r="I611" s="8" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="J611" s="8" t="n">
+        <v>-10.3171</v>
+      </c>
       <c r="K611" s="6" t="inlineStr">
         <is>
           <t>Üretici imalatı</t>
@@ -26830,7 +26830,7 @@
       </c>
       <c r="L611" s="6" t="inlineStr">
         <is>
-          <t>BIST TUM-100, BIST SINAI, BIST TÜM, BIST KİMYA PETROL PLASTİK, BIST HALKA ARZ, BIST KATILIM TÜM, BIST ANA, BIST TEKİRDAĞ</t>
+          <t>BIST TUM-100, BIST TÜM, BIST HOLDING VE YATIRIM, BIST MALİ, BIST KATILIM 100, BIST KATILIM TÜM, BIST YILDIZ, BIST KATILIM 50, BIST KONYA</t>
         </is>
       </c>
       <c r="M611" s="6" t="inlineStr"/>
@@ -26857,7 +26857,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>06.05.2026 16:30</t>
+          <t>06.05.2026 16:59</t>
         </is>
       </c>
     </row>

</xml_diff>